<commit_message>
docs: survey xlsx - drop legend sheet and applications group (93 papers)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QUQHKThf7Jqhp8h8pyLsF
</commit_message>
<xml_diff>
--- a/docs/tabpfn_papers_survey.xlsx
+++ b/docs/tabpfn_papers_survey.xlsx
@@ -8,10 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TabPFN survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="범례" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TabPFN survey'!$A$1:$O$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TabPFN survey'!$A$1:$O$94</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,11 +35,8 @@
     <font>
       <sz val="9"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
   </fonts>
-  <fills count="13">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -89,11 +85,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E6F7FB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00F0F4E8"/>
       </patternFill>
     </fill>
@@ -129,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -164,20 +155,6 @@
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -543,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O100"/>
+  <dimension ref="A1:O94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5741,53 +5718,57 @@
     <row r="72" ht="95" customHeight="1">
       <c r="A72" s="10" t="inlineStr">
         <is>
-          <t>TabPFN-Credit</t>
+          <t>TabRep-Survey</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Foundation Models for Credit Risk Prediction: A Game Changer?</t>
-        </is>
-      </c>
-      <c r="C72" s="4" t="inlineStr"/>
+          <t>Representation Learning for Tabular Data: A Comprehensive Survey</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/LAMDA-Tabular/Tabular-Survey</t>
+        </is>
+      </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>신용위험 모형(부도확률·부도시손실률)은 규제 산업에서 여전히 전통적 기법이 지배적인데, 표 형식 파운데이션 모델의 사전지식이 신용위험 평가를 개선할 수 있는지 대규모로 검증할 필요가 있었다.</t>
+          <t>tabular 딥러닝 방법이 폭증하고 TabPFN류 foundation model까지 등장했으나, 일반화 능력 관점에서 전체 지형을 정리한 최신 서베이가 부족했다.</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>PD(부도확률)와 LGD(부도시손실률) 모델링에서 표 형식 파운데이션 모델을 기존 기법과 체계적으로 벤치마크하는 것.</t>
+          <t>tabular 표현학습 방법을 일반화 능력 기준의 3단계 체계로 종합 정리하는 것.</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>TabPFN 계열의 사전학습 표 형식 파운데이션 모델을 하이퍼파라미터 튜닝 없이 다수의 신용 데이터셋에 적용한다. PD(분류)와 LGD(회귀) 과제 각각에 대해 확립된 신용평가 기법들과 다양한 실험 조건(특히 소규모 데이터 상황)에서 비교한다.</t>
+          <t>방법론을 단일 분포용 specialized 모델, 사전학습-파인튜닝형 transferable 모델, 파인튜닝 없이 쓰는 general foundation 모델(TabPFN류 포함)의 3범주로 조직화한다. specialized 모델에 대해 특징·샘플·목적함수 축의 계층적 분류체계를 제시하고, 앙상블·개방환경 ML·멀티모달·테이블 이해까지 확장 주제를 다룬다.</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>다수의 신용위험 데이터셋(PD 및 LGD 모델링용; 초록에 개별 명칭 미기재)</t>
+          <t>해당 없음 (서베이; 주요 벤치마크와 DNN 사용의 장단점 정리)</t>
         </is>
       </c>
       <c r="H72" s="4" t="inlineStr">
         <is>
-          <t>신용평가 분야의 확립된 통계·머신러닝 기법들</t>
+          <t>해당 없음 (specialized/transferable/general 3범주 간 정성적 비교)</t>
         </is>
       </c>
       <c r="I72" s="4" t="inlineStr">
         <is>
-          <t>데이터셋·과제(PD/LGD)·실험 조건 전반의 벤치마크, 소규모 데이터 시나리오 분석, 튜닝 비용 비교</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="J72" s="4" t="inlineStr">
         <is>
-          <t>PD (classification) and LGD (regression) predictive performance</t>
+          <t>N/A (survey)</t>
         </is>
       </c>
       <c r="K72" s="4" t="inlineStr">
         <is>
-          <t>파운데이션 모델이 데이터셋과 과제 전반에서 대체로 경쟁 기법을 능가했으며, 특히 소규모 데이터 상황에서 개선 폭이 두드러졌다. 하이퍼파라미터 튜닝 없이도 강한 성능을 내 계산 부담을 줄였다.</t>
+          <t>specialized → transferable → general(foundation)로 이어지는 3단계 일반화 스펙트럼 분류체계를 제시해 TabPFN 계열과 CARTE·TP-BERTa류 전이 모델을 하나의 지도 위에 배치했다. 특징·샘플·목적함수 축의 계층적 taxonomy와 함께 GitHub에 논문 목록을 지속 갱신 중이다.</t>
         </is>
       </c>
       <c r="L72" s="4" t="inlineStr">
@@ -5797,210 +5778,222 @@
       </c>
       <c r="M72" s="4" t="inlineStr">
         <is>
-          <t>arXiv (cs.LG)</t>
+          <t>arXiv</t>
         </is>
       </c>
       <c r="N72" s="4" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="O72" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2605.18147</t>
+          <t>https://arxiv.org/pdf/2504.16109</t>
         </is>
       </c>
     </row>
     <row r="73" ht="95" customHeight="1">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>TabPFN-Ins</t>
+          <t>TabSTAR</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Is TabPFN the Silver Bullet for Insurance Pricing?</t>
-        </is>
-      </c>
-      <c r="C73" s="4" t="inlineStr"/>
+          <t>TabSTAR: A Tabular Foundation Model for Tabular Data with Text Fields</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/alanarazi7/TabSTAR</t>
+        </is>
+      </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>비생명(손해)보험 요율산정은 전통적으로 GLM과 그래디언트 부스팅에 의존해 왔는데, 합성 데이터로 사전학습된 표 형식 파운데이션 모델이 이를 대체할 수 있는지 검증된 바 없었다.</t>
+          <t>tabular 딥러닝은 GBDT에 뒤처져 왔고, TabPFN류도 자유 텍스트 특징을 가진 테이블에서는 의미 정보를 충분히 활용하지 못한다. 텍스트 특징이 있는 테이블에서의 전이학습이 목표 공백이다.</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>자동차보험 요율산정에 대한 TabPFN의 최초 실증 평가를 수행하는 것.</t>
+          <t>데이터셋 특화 파라미터 없이 텍스트 특징 테이블에 전이 가능한 tabular foundation model(TabSTAR)을 만드는 것.</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>합성 데이터 사전학습과 인컨텍스트 학습으로 데이터셋별 적합 과정 없이 추론하는 TabPFN을 보험 클레임 예측 파이프라인에 적용한다. 동일 데이터·동일 분할에서 GLM 및 XGBoost와 직접 비교하고, 학습 표본 크기에 대한 민감도를 분석한다.</t>
+          <t>사전학습된 텍스트 인코더를 unfrozen 상태로 학습하며 타깃 인식(semantically target-aware) 표현을 만들고, target token을 입력해 태스크별 임베딩을 학습한다. 350개 tabular 데이터셋(분류 253, 회귀 97)으로 사전학습한 뒤 다운스트림별 파인튜닝한다.</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>공개 자동차 제3자 배상책임(MTPL) 보험 데이터셋 2종</t>
+          <t>사전학습 350개 데이터셋; 평가는 AutoML Multimodal Benchmark·CARTE 벤치마크 등에서 모은 텍스트 특징 포함 50개 데이터셋(데이터셋당 10회 분할, 총 500 런)</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>GLM(일반화선형모형), XGBoost</t>
+          <t>CatBoost(tuned), TabM(tuned), TabPFN-v2, CARTE 등 GBDT·tabular DNN·tabular FM</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>두 데이터셋에서의 요율산정 예측 성능 비교, 추론 시간 측정, 학습 세트 크기 변화에 따른 성능 민감도 실험</t>
+          <t>10K 예제 제한/무제한(100K 상한) 두 조건의 분류·회귀 평가, 사전학습 데이터셋 수에 대한 scaling law 분석, head-to-head 승률 분석</t>
         </is>
       </c>
       <c r="J73" s="4" t="inlineStr">
         <is>
-          <t>Pricing predictive performance and inference time (abstract-level; standard actuarial accuracy measures)</t>
+          <t>AUROC (classification), R2 (regression), normalized score</t>
         </is>
       </c>
       <c r="K73" s="4" t="inlineStr">
         <is>
-          <t>TabPFN은 확립된 베이스라인(GLM·XGBoost)을 일관되게 능가하지 못했고 추론 시간이 상당히 길었으며 학습 표본 크기에 민감했다. 데이터가 희소한 상황에서는 유망하지만 현행 보험계리 기법의 대체재로는 아직 부적합하다고 결론지었다.</t>
+          <t>10K 조건 분류에서 normalized score 0.83으로 TabM-Tuned(0.73), CatBoost-Tuned(0.69), TabPFN-v2(0.67)를 앞섰고, TabPFN-v2 상대 11개 중 8개 데이터셋에서 승리했다. 무제한 조건에서도 0.84로 선두였으며, 사전학습 데이터셋 수에 대한 scaling law가 관찰됐다.</t>
         </is>
       </c>
       <c r="L73" s="4" t="inlineStr">
         <is>
-          <t>MTPL 2종 데이터셋에 한정된 평가이며, 대규모 포트폴리오·다양한 보험 상품으로의 일반화는 확인되지 않았다.</t>
+          <t>회귀에서는 경쟁력은 있으나 GBDT가 여전히 우세</t>
         </is>
       </c>
       <c r="M73" s="4" t="inlineStr">
         <is>
-          <t>arXiv (q-fin.RM)</t>
+          <t>NeurIPS 2025</t>
         </is>
       </c>
       <c r="N73" s="4" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="O73" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2605.22892</t>
+          <t>https://arxiv.org/pdf/2505.18125</t>
         </is>
       </c>
     </row>
     <row r="74" ht="95" customHeight="1">
       <c r="A74" s="10" t="inlineStr">
         <is>
-          <t>TFM-Mol</t>
+          <t>CARTE</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Tabular foundation models for in-context prediction of molecular properties</t>
-        </is>
-      </c>
-      <c r="C74" s="4" t="inlineStr"/>
+          <t>CARTE: Pretraining and Transfer for Tabular Learning</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/soda-inria/carte</t>
+        </is>
+      </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>신약개발·촉매·공정설계의 분자 물성 예측은 소규모 데이터에 제약되며, 분자 파운데이션 모델은 과제별 파인튜닝과 ML 전문성이 필요함에도 고전 베이스라인을 넘지 못하는 경우가 많다.</t>
+          <t>테이블 간 전이는 entity matching·schema matching 같은 데이터 통합 작업을 요구해 왔다. 컬럼 대응 없이도 서로 다른 테이블 간 지식을 전이할 수 있는 구조가 필요하다.</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>저·중규모 데이터 영역에서 표 형식 파운데이션 모델의 인컨텍스트 학습이 분자 물성 예측의 정확하고 저비용인 대안이 되는지 평가하는 것.</t>
+          <t>테이블 행을 그래프로 표현해 스키마 매칭 없이 사전학습·전이가 가능한 tabular 신경망(CARTE)을 만드는 것.</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>분자를 고정(frozen) 분자 파운데이션 모델 임베딩(CheMeleon 등), 고전 기술자(RDKit2d, Mordred), 지문(fingerprint)으로 표현해 표 형식 입력으로 변환한 뒤, TabPFN 계열 TFM이 파인튜닝 없이 인컨텍스트로 물성을 예측한다. 표현 방식별 성능을 체계적으로 비교한다.</t>
+          <t>각 행을 star graph로 표현하고 셀 값·컬럼명을 문자열 임베딩으로 개방 어휘(open vocabulary) 처리한 뒤, graph-attentional network로 컬럼명·이웃 셀 문맥을 반영한 표현을 학습한다. YAGO3 지식베이스(630만 엔티티, 1,810만 트리플)로 사전학습한 후 다운스트림 테이블에 파인튜닝하며, 매칭되지 않은 컬럼을 가진 테이블 간 공동 학습도 지원한다.</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>표준 제약 벤치마크(MoleculeACE 30개 과제 포함)와 화학공학 데이터셋</t>
+          <t>YAGO3 지식그래프(사전학습), Kaggle 등에서 수집한 51개 tabular 데이터셋(회귀 40, 분류 11)</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr">
         <is>
-          <t>파인튜닝된 분자 파운데이션 모델, 고전 기술자·지문 기반 모델</t>
+          <t>CatBoost·XGBoost 등 트리 모델과 TabPFN을 포함한 42개 베이스라인</t>
         </is>
       </c>
       <c r="I74" s="4" t="inlineStr">
         <is>
-          <t>저·중규모 데이터 영역에서의 벤치마크 평가, 분자 표현(임베딩 vs 기술자 vs 지문)별 비교, 계산 비용 분석, 공학 데이터로의 전이 검증</t>
+          <t>샘플 수를 변화시킨 single-table 학습 곡선, 결측치 강건성, 관련 주제 테이블 간 multi-table 전이 실험</t>
         </is>
       </c>
       <c r="J74" s="4" t="inlineStr">
         <is>
-          <t>Win rate over baselines, regression accuracy, computational cost</t>
+          <t>AUROC (classification), R2 (regression), normalized score, critical-difference rank</t>
         </is>
       </c>
       <c r="K74" s="4" t="inlineStr">
         <is>
-          <t>TFM과 CheMeleon 임베딩 결합 시 MoleculeACE 30개 과제에서 최대 100% 승률을 달성했으며, 파인튜닝 대비 계산 비용을 줄이면서 우수한 예측 성능을 보였다. 분자 표현 선택이 TFM 성능의 핵심 결정 요인으로 나타났다.</t>
+          <t>51개 데이터셋에서 42개 베이스라인 대비 평균 순위 1위로 최상의 트리 모델(CatBoost 등)을 능가했고, 특히 고카디널리티 문자열 컬럼이 많은 데이터에서 강했다. 매칭되지 않은 소스 테이블을 추가할수록 중앙값 성능이 오르고 분산이 줄어 cross-table 전이 이득을 입증했다.</t>
         </is>
       </c>
       <c r="L74" s="4" t="inlineStr">
         <is>
-          <t>저·중규모 데이터 영역에 평가가 한정되며, 분자 표현에 따라 성능 편차가 크다.</t>
+          <t>명시 없음</t>
         </is>
       </c>
       <c r="M74" s="4" t="inlineStr">
         <is>
-          <t>arXiv (cs.LG, physics.chem-ph)</t>
+          <t>ICML 2024</t>
         </is>
       </c>
       <c r="N74" s="4" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="O74" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2604.16123</t>
+          <t>https://arxiv.org/pdf/2402.16785</t>
         </is>
       </c>
     </row>
     <row r="75" ht="95" customHeight="1">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>TFM-Surv</t>
+          <t>CM2</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Tabular Foundation Models Can Do Survival Analysis</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr"/>
+          <t>Towards Cross-Table Masked Pretraining for Web Data Mining</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/Chao-Ye/CM2</t>
+        </is>
+      </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>생존분석은 우측 중도절단(right censoring) 처리 때문에 전용 모델이 필요해, 표 형식 파운데이션 모델의 인컨텍스트 학습 이점을 그대로 활용하기 어려웠다.</t>
+          <t>웹에는 방대한 이질적 테이블이 있으나 기존 tabular 사전학습은 단일 테이블 수준에 머물러 NLP의 'BERT moment'에 해당하는 돌파구가 없었다.</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>생존분석을 이진 분류의 연속으로 재정식화하여 기성 표 형식 파운데이션 모델이 별도 훈련 없이 생존분석을 수행하게 하는 것.</t>
+          <t>웹 규모의 이질적 테이블 코퍼스에 대한 masked pretraining으로 범용 tabular 표현을 학습하는 것.</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>사건 시각을 이산화하여 정적·동적 생존분석을 시점별 이진 분류 문제의 나열로 변환하고, 중도절단 관측치는 해당 시점의 결측 레이블로 자연스럽게 처리한다. 이산시간 위험률(hazard)이 아니라 누적 실패 확률을 직접 모델링하여 이산화 선택에 대한 강건성을 확보하고, TabPFN류 모델의 인컨텍스트 학습으로 예측한다.</t>
+          <t>이질적 테이블을 통일 인코딩하는 semantic-aware tabular neural network를 설계하고, NLP의 MLM을 테이블에 맞게 변형한 prompt Masked Table Modeling(pMTM) 목적함수로 사전학습한다. OpenML·UCI·Kaggle 등에서 수집한 약 2,000개 테이블·4,600만 샘플 규모의 OpenTabs 코퍼스를 구축해 사용한다.</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>실제 생존분석 데이터셋 48개(정적 43개, 동적 5개 벤치마크)</t>
+          <t>OpenTabs(약 2,000개 테이블, 4,600만 샘플) 사전학습; 다운스트림 분류 16개, 회귀 6개, 이상탐지·결측치 대체 데이터셋</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>고전 생존분석 기법 및 딥러닝 생존모델</t>
+          <t>FT-Transformer 등 tabular 딥러닝, 트리 계열, 기존 tabular 사전학습 방법</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>48개 데이터셋에서의 정적·동적 생존분석 벤치마크, 이산화 방식에 대한 강건성 분석, 다중 생존 지표에 대한 평균 성능 비교</t>
+          <t>supervised 파인튜닝, few-shot(5-shot 등), 이상탐지·결측 대체 등 다양한 다운스트림 전이 실험</t>
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr">
         <is>
-          <t>Multiple survival analysis metrics (concordance/calibration-type; averaged across benchmarks)</t>
+          <t>AUC (classification), RMSE (regression), F1 (anomaly detection)</t>
         </is>
       </c>
       <c r="K75" s="4" t="inlineStr">
         <is>
-          <t>기성 표 형식 파운데이션 모델이 명시적 생존 훈련 없이도 43개 정적·5개 동적 벤치마크에서 다중 생존 지표 평균으로 고전 및 딥러닝 베이스라인을 능가했다. 누적 실패 확률 직접 모델링이 이산화 선택에 강건함을 보였다.</t>
+          <t>16개 분류 데이터셋 중 12개에서 모든 베이스라인을 상회하며 SOTA 평균 성능을 달성했고, few-shot(특히 5-shot)에서 from-scratch 대비 사전학습 이득이 가장 컸다. 기존 연구가 10~52개 테이블로 사전학습한 데 비해 약 2,000개 테이블로 규모를 확장했다.</t>
         </is>
       </c>
       <c r="L75" s="4" t="inlineStr">
@@ -6010,378 +6003,374 @@
       </c>
       <c r="M75" s="4" t="inlineStr">
         <is>
-          <t>arXiv (cs.LG)</t>
+          <t>WWW 2024</t>
         </is>
       </c>
       <c r="N75" s="4" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="O75" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2601.22259</t>
+          <t>https://arxiv.org/pdf/2307.04308</t>
         </is>
       </c>
     </row>
     <row r="76" ht="95" customHeight="1">
       <c r="A76" s="10" t="inlineStr">
         <is>
-          <t>TabPFN-RNAseq</t>
+          <t>GTL</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>The Limitations of TabPFN for High-Dimensional RNA-seq Analysis</t>
-        </is>
-      </c>
-      <c r="C76" s="4" t="inlineStr"/>
+          <t>From Supervised to Generative: A Novel Paradigm for Tabular Deep Learning with Large Language Models</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/microsoft/Industrial-Foundation-Models</t>
+        </is>
+      </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>전사체(RNA-seq) 데이터는 유전자 수만 개의 고차원·소표본 구조인데, TabPFN의 입력 특징 제한(500개)과 고차원 확장 시의 거동이 유전체 분석 실무에 적합한지 검증되지 않았다.</t>
+          <t>기존 tabular 딥러닝은 지식 전이, 소수 데이터 일반화, 지시 따르기 등 범용 모델 요구를 충족하지 못한다. LLM의 zero-shot 일반화와 in-context learning을 tabular 예측에 이식하려 한다.</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>고차원 RNA-seq 분석에서 TabPFN 및 그 변형들의 성능 한계를 실증적으로 규명하는 것.</t>
+          <t>다양한 tabular 데이터에 대한 생성적 continued pretraining(GTL)으로 LLM에 범용 tabular 예측 능력을 부여하는 것.</t>
         </is>
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>대규모 RNA-seq 데이터에서 TabPFN(및 고차원 처리를 위한 구조 변형)을 회귀·분류 과제에 적용한다. 특징 수를 500개로 제한한 조건과 전체 특징을 사용하는 조건에서 고전 모델과 성능을 교차 비교하고, 메타데이터 기반 서브그룹핑 등 배치 전략을 분석한다.</t>
+          <t>테이블을 지시·특징·타깃이 포함된 텍스트 템플릿으로 변환해 LLaMA-2를 384개 공개 데이터셋 위에서 생성적(next-token) 방식으로 continued pretraining한다. 프롬프트 기반 zero-shot과 in-context 예시를 통한 few-shot 예측을 하나의 생성 패러다임으로 통일하고, 수렴·스케일링 거동과 데이터 템플릿 영향을 분석한다.</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>Age-ARCHS4(ARCHS4 기반 연령 회귀, 57,873 샘플 × 10,000 유전자), IBD 분류 데이터(크론병·궤양성대장염 포함, 2,490 샘플 × 10,000 유전자)</t>
+          <t>384개 공개 tabular 데이터셋(분류·회귀)</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr">
         <is>
-          <t>Random Forest, XGBoost, 나이브 베이스라인</t>
+          <t>전통적 지도학습 tabular 방법들과 GPT-4 등 범용 LLM</t>
         </is>
       </c>
       <c r="I76" s="4" t="inlineStr">
         <is>
-          <t>500 특징 제한 조건 vs 전체 특징 조건 비교 실험, 고차원 처리용 TabPFN 변형 평가, 메타데이터 서브그룹핑 배치 전략 검증</t>
+          <t>zero-shot·in-context learning 평가, 스케일링/수렴 분석, 데이터 템플릿 ablation</t>
         </is>
       </c>
       <c r="J76" s="4" t="inlineStr">
         <is>
-          <t>Regression error (age prediction) and classification performance (IBD)</t>
+          <t>zero-shot / in-context accuracy (classification), regression error</t>
         </is>
       </c>
       <c r="K76" s="4" t="inlineStr">
         <is>
-          <t>특징을 500개로 제한하면 TabPFN이 RF·XGBoost를 능가하지만, 고전 모델이 10,000 유전자 전체를 쓰는 조건에서는 모든 TabPFN 변형이 나이브 베이스라인조차 일관되게 하회했다. 고차원 대응 구조 변형은 오히려 성능을 저하시켰고, 메타데이터 기반 서브그룹핑이 가장 효과적인 활용 전략으로 나타났다.</t>
+          <t>GTL로 강화된 LLaMA-2는 384개 데이터셋 실험에서 파인튜닝 없이 zero-shot·ICL 성능이 전통 방법을 능가했고, 일부 태스크에서는 GPT-4에 필적했다.</t>
         </is>
       </c>
       <c r="L76" s="4" t="inlineStr">
         <is>
-          <t>동료심사 전 bioRxiv 프리프린트이며, 평가가 두 개의 RNA-seq 과제에 한정된다.</t>
+          <t>명시 없음</t>
         </is>
       </c>
       <c r="M76" s="4" t="inlineStr">
         <is>
-          <t>bioRxiv</t>
+          <t>KDD 2024</t>
         </is>
       </c>
       <c r="N76" s="4" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="O76" s="4" t="inlineStr">
         <is>
-          <t>https://www.biorxiv.org/content/10.1101/2025.08.15.670537v1.full.pdf</t>
+          <t>https://arxiv.org/pdf/2310.07338</t>
         </is>
       </c>
     </row>
     <row r="77" ht="95" customHeight="1">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>TabPFN-Stat</t>
+          <t>LLM-TabSurvey</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>TabPFN: One Model to Rule Them All?</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/qinglong-tian/tabpfn_study</t>
-        </is>
-      </c>
+          <t>Large Language Models(LLMs) on Tabular Data: Prediction, Generation, and Understanding -- A Survey</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr"/>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>TabPFN이 근사 베이지안 추론을 수행한다는 관점에서, 표준 예측을 넘어 통계학의 다양한 추정 문제에 기성 모델을 그대로 활용할 수 있는지가 미지수였다.</t>
+          <t>LLM을 tabular 예측·생성·이해에 적용하는 연구가 급증했으나 핵심 기법·메트릭·데이터셋·미해결 과제를 아우르는 종합 정리가 없었다.</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>TabPFN을 근사 베이지안 추론으로 해석하고 준지도 추정·공변량 이동·처치효과 추정 등 통계 응용에서의 성능을 규명하는 것.</t>
+          <t>tabular 데이터에 대한 LLM 활용(예측·생성·이해)을 체계적으로 분류·정리하는 것.</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>TabPFN의 인컨텍스트 예측을 근사 베이지안 추론으로 정식화하고, 이를 준지도 모수 추정(선형·로지스틱·분위수 회귀), 이질적 처치효과(CATE) 추정, 공변량 이동 하 예측, 데이터 생성·밀도 추정에 기성(off-the-shelf) 상태로 적용한다. 비모수·모수 구조에 대한 동시 적응성을 이론·실험으로 분석한다.</t>
+          <t>LLM 기반 tabular 모델링을 예측(prediction), 데이터 생성(generation), 이해(table QA·comprehension)의 3개 축으로 나눠 직렬화·프롬프트·파인튜닝 등 기법을 분류한다. 각 축의 데이터셋·메트릭 분류체계를 제공하고 연구 공백과 향후 방향을 제시한다.</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>시뮬레이션 데이터 및 각 통계 과제별 벤치마크 데이터(준지도 추정, CATE, 공변량 이동 실험)</t>
+          <t>해당 없음 (서베이; 각 축별 공개 데이터셋·벤치마크 분류 제공)</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>LASSO 등 정통 통계 추정량, 전용 준지도·CATE·공변량 이동 기법, 가우시안 프로세스 회귀</t>
+          <t>해당 없음 (기존 방법론 간 정성적 비교·분류)</t>
         </is>
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>준지도 모수 추정 실험(Study I), CATE 추정(Study II), 공변량 이동 하 예측(Study III), 회귀·분류에서의 적응성 분석 및 불확실성 정량화 비교</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="J77" s="4" t="inlineStr">
         <is>
-          <t>Estimation error / MSE for parameter and CATE estimation, prediction accuracy under covariate shift</t>
+          <t>N/A (survey)</t>
         </is>
       </c>
       <c r="K77" s="4" t="inlineStr">
         <is>
-          <t>기성 TabPFN이 준지도 추정·공변량 이동·처치효과 추정에서 전용 기법을 능가하는 경우가 있었고, 모형 가정이 올바르게 특정된 상황에서도 LASSO를 능가하기도 했다. 비모수 구조와 모수 구조에 동시에 적응하는 성질을 보였다.</t>
+          <t>41페이지, 8개 표 분량으로 LLM 기반 tabular 예측·생성·이해 기법과 데이터셋·메트릭의 분류체계를 정리했고, 직렬화 방식·파인튜닝 전략별 장단점과 미해결 과제(수치 표현, 대규모 테이블 처리 등)를 도출했다. TabLLM·GTL류 LLM 기반 예측 계열의 표준 참조 서베이로 자리잡았다.</t>
         </is>
       </c>
       <c r="L77" s="4" t="inlineStr">
         <is>
+          <t>빠르게 발전하는 분야 특성상 2024년 이후 모델은 미포함</t>
+        </is>
+      </c>
+      <c r="M77" s="4" t="inlineStr">
+        <is>
+          <t>TMLR 2024</t>
+        </is>
+      </c>
+      <c r="N77" s="4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="O77" s="4" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2402.17944</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="95" customHeight="1">
+      <c r="A78" s="10" t="inlineStr">
+        <is>
+          <t>LTM-Position</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Why Tabular Foundation Models Should Be a Research Priority</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr"/>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>텍스트·이미지 foundation model에 연구 자원이 쏠리는 동안 여러 분야의 지배적 데이터 양식인 tabular 데이터는 규모·역량 면에서 크게 뒤처져 있다.</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>Large Tabular Model(LTM) 개발을 ML 커뮤니티의 우선 연구 과제로 제안하는 것.</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>포지션 논문으로서 tabular 도메인의 연구 공백을 진단하고 LTM 개념을 정의한다. few-shot tabular 모델, 데이터 사이언스 자동화, OOD 합성 데이터, 다학제 과학 발견 등 LTM의 파급 효과와 연구 로드맵(데이터, 아키텍처, 평가 과제)을 논한다.</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>해당 없음 (포지션 논문)</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>해당 없음</t>
+        </is>
+      </c>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t>해당 없음</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t>N/A (position paper)</t>
+        </is>
+      </c>
+      <c r="K78" s="4" t="inlineStr">
+        <is>
+          <t>tabular 데이터가 다수 분야의 지배적 양식임에도 연구 관심이 미미함을 지적하고, 단일 데이터셋 고립 분석에서 관련 데이터셋 맥락화로의 전환을 LTM의 핵심 가치로 제시했다. TabPFN류 초기 시도를 넘어서는 스케일업 필요성을 논증해 이후 tabular FM 연구의 방향 설정에 널리 인용된다.</t>
+        </is>
+      </c>
+      <c r="L78" s="4" t="inlineStr">
+        <is>
+          <t>실험적 검증이 없는 포지션 논문</t>
+        </is>
+      </c>
+      <c r="M78" s="4" t="inlineStr">
+        <is>
+          <t>ICML 2024 (position paper)</t>
+        </is>
+      </c>
+      <c r="N78" s="4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="O78" s="4" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2405.01147</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="95" customHeight="1">
+      <c r="A79" s="10" t="inlineStr">
+        <is>
+          <t>TabuLa-8B</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Large Scale Transfer Learning for Tabular Data via Language Modeling</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/mlfoundations/rtfm</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>언어·비전에서 foundation model이 태스크별 모델 개발을 대체했지만 tabular 도메인에는 그런 전이학습 패러다임이 부재하다. 웹 규모 테이블 코퍼스로 LLM을 학습하면 보지 못한 테이블에 대한 zero/few-shot 예측이 가능한지 검증한다.</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>TabLib 코퍼스로 파인튜닝한 LLM(TabuLa-8B)으로 대규모 tabular 전이학습(zero/few-shot 예측)을 실현하는 것.</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>TabLib에서 필터링·품질 관리를 거쳐 400만여 개 테이블·21억 행의 학습 데이터(T4)를 추출하고, Llama 3-8B를 tabular 예측(분류·구간화 회귀)용으로 파인튜닝한다. 행 단위 예측에 맞춘 novel packing·attention 마스킹 기법을 도입한다.</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>TabLib 유래 T4 코퍼스(2.1B 행, 4M+ 테이블) 학습; 329개 데이터셋 평가 스위트</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>XGBoost, TabPFN 등 SOTA tabular 예측 모델(타깃 데이터로 명시적으로 학습된 조건 포함)</t>
+        </is>
+      </c>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>미학습 테이블에 대한 zero-shot 예측, 1~32 shot few-shot(타깃 파인튜닝 없음) 비교, 상대 모델에 최대 16배 데이터를 준 조건 비교</t>
+        </is>
+      </c>
+      <c r="J79" s="4" t="inlineStr">
+        <is>
+          <t>zero-shot / few-shot accuracy (percentage points vs. random and baselines)</t>
+        </is>
+      </c>
+      <c r="K79" s="4" t="inlineStr">
+        <is>
+          <t>329개 데이터셋에서 zero-shot 정확도가 무작위 추측보다 15pp 이상 높았는데 이는 XGBoost·TabPFN 등 기존 모델로는 불가능한 능력이다. 1~32 shot에서는 동량 또는 최대 16배 많은 데이터로 학습된 XGBoost·TabPFN보다 5~15pp 더 정확했다.</t>
+        </is>
+      </c>
+      <c r="L79" s="4" t="inlineStr">
+        <is>
           <t>명시 없음</t>
         </is>
       </c>
-      <c r="M77" s="4" t="inlineStr">
-        <is>
-          <t>arXiv; Journal of the American Statistical Association</t>
-        </is>
-      </c>
-      <c r="N77" s="4" t="n">
-        <v>2025</v>
-      </c>
-      <c r="O77" s="4" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/pdf/2505.20003</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="95" customHeight="1">
-      <c r="A78" s="11" t="inlineStr">
-        <is>
-          <t>TabRep-Survey</t>
-        </is>
-      </c>
-      <c r="B78" s="4" t="inlineStr">
-        <is>
-          <t>Representation Learning for Tabular Data: A Comprehensive Survey</t>
-        </is>
-      </c>
-      <c r="C78" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/LAMDA-Tabular/Tabular-Survey</t>
-        </is>
-      </c>
-      <c r="D78" s="4" t="inlineStr">
-        <is>
-          <t>tabular 딥러닝 방법이 폭증하고 TabPFN류 foundation model까지 등장했으나, 일반화 능력 관점에서 전체 지형을 정리한 최신 서베이가 부족했다.</t>
-        </is>
-      </c>
-      <c r="E78" s="4" t="inlineStr">
-        <is>
-          <t>tabular 표현학습 방법을 일반화 능력 기준의 3단계 체계로 종합 정리하는 것.</t>
-        </is>
-      </c>
-      <c r="F78" s="4" t="inlineStr">
-        <is>
-          <t>방법론을 단일 분포용 specialized 모델, 사전학습-파인튜닝형 transferable 모델, 파인튜닝 없이 쓰는 general foundation 모델(TabPFN류 포함)의 3범주로 조직화한다. specialized 모델에 대해 특징·샘플·목적함수 축의 계층적 분류체계를 제시하고, 앙상블·개방환경 ML·멀티모달·테이블 이해까지 확장 주제를 다룬다.</t>
-        </is>
-      </c>
-      <c r="G78" s="4" t="inlineStr">
-        <is>
-          <t>해당 없음 (서베이; 주요 벤치마크와 DNN 사용의 장단점 정리)</t>
-        </is>
-      </c>
-      <c r="H78" s="4" t="inlineStr">
-        <is>
-          <t>해당 없음 (specialized/transferable/general 3범주 간 정성적 비교)</t>
-        </is>
-      </c>
-      <c r="I78" s="4" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="J78" s="4" t="inlineStr">
-        <is>
-          <t>N/A (survey)</t>
-        </is>
-      </c>
-      <c r="K78" s="4" t="inlineStr">
-        <is>
-          <t>specialized → transferable → general(foundation)로 이어지는 3단계 일반화 스펙트럼 분류체계를 제시해 TabPFN 계열과 CARTE·TP-BERTa류 전이 모델을 하나의 지도 위에 배치했다. 특징·샘플·목적함수 축의 계층적 taxonomy와 함께 GitHub에 논문 목록을 지속 갱신 중이다.</t>
-        </is>
-      </c>
-      <c r="L78" s="4" t="inlineStr">
+      <c r="M79" s="4" t="inlineStr">
+        <is>
+          <t>NeurIPS 2024</t>
+        </is>
+      </c>
+      <c r="N79" s="4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="O79" s="4" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2406.12031</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="95" customHeight="1">
+      <c r="A80" s="10" t="inlineStr">
+        <is>
+          <t>TP-BERTa</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Making Pre-trained Language Models Great on Tabular Prediction</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/jyansir/tp-berta</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>이미지·언어에서 확립된 전이학습이 tabular 예측에서는 미활용 상태이며, LM을 그대로 쓰면 수치 특징 값을 제대로 표현하지 못한다. 수치값의 크기 정보를 LM 토큰 공간에 이식하는 것이 관건이다.</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>수치 특징을 다룰 수 있게 특화 사전학습한 언어 모델(TP-BERTa)로 tabular 예측에서 GBDT급 성능을 내는 것.</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>수치값을 상대적 크기 기반 이산 토큰으로 바꾸는 relative magnitude tokenization(RMT)으로 수치를 LM 어휘에 통합한다. intra-feature attention(IFA)으로 특징명과 값을 결합해 특징 단위 표현을 만들고, RoBERTa를 101개 이진 분류 + 101개 회귀 데이터셋(약 1천만 샘플)으로 사전학습한다.</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>사전학습 202개 데이터셋(약 10M 샘플), 다운스트림 145개 데이터셋(이진 분류 80개, 회귀 65개)</t>
+        </is>
+      </c>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>tuned XGBoost/CatBoost 등 GBDT, FT-Transformer 등 tabular DNN, 기존 LM 기반 tabular 접근</t>
+        </is>
+      </c>
+      <c r="I80" s="4" t="inlineStr">
+        <is>
+          <t>default/tuned 설정별 평균 순위 비교, 범주형 특징 비중에 따른 성능 분석, RMT/IFA ablation</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="inlineStr">
+        <is>
+          <t>AUC (binary classification), RMSE (regression), average rank</t>
+        </is>
+      </c>
+      <c r="K80" s="4" t="inlineStr">
+        <is>
+          <t>145개 다운스트림에서 default 설정 기준 평균 순위 5.8로 tuned XGBoost(6.2), tuned CatBoost(5.9)와 대등한 GBDT급 성능을 달성했다. 범주형 특징이 우세한 데이터셋에서는 순위 4.4로 tuned CatBoost(7.1)를 크게 앞섰고, RMT 인코딩은 기존 LM 인코딩 대비 AUC를 최대 12.45% 개선했다.</t>
+        </is>
+      </c>
+      <c r="L80" s="4" t="inlineStr">
         <is>
           <t>명시 없음</t>
         </is>
       </c>
-      <c r="M78" s="4" t="inlineStr">
-        <is>
-          <t>arXiv</t>
-        </is>
-      </c>
-      <c r="N78" s="4" t="n">
-        <v>2025</v>
-      </c>
-      <c r="O78" s="4" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/pdf/2504.16109</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="95" customHeight="1">
-      <c r="A79" s="11" t="inlineStr">
-        <is>
-          <t>TabSTAR</t>
-        </is>
-      </c>
-      <c r="B79" s="4" t="inlineStr">
-        <is>
-          <t>TabSTAR: A Tabular Foundation Model for Tabular Data with Text Fields</t>
-        </is>
-      </c>
-      <c r="C79" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/alanarazi7/TabSTAR</t>
-        </is>
-      </c>
-      <c r="D79" s="4" t="inlineStr">
-        <is>
-          <t>tabular 딥러닝은 GBDT에 뒤처져 왔고, TabPFN류도 자유 텍스트 특징을 가진 테이블에서는 의미 정보를 충분히 활용하지 못한다. 텍스트 특징이 있는 테이블에서의 전이학습이 목표 공백이다.</t>
-        </is>
-      </c>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>데이터셋 특화 파라미터 없이 텍스트 특징 테이블에 전이 가능한 tabular foundation model(TabSTAR)을 만드는 것.</t>
-        </is>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
-        <is>
-          <t>사전학습된 텍스트 인코더를 unfrozen 상태로 학습하며 타깃 인식(semantically target-aware) 표현을 만들고, target token을 입력해 태스크별 임베딩을 학습한다. 350개 tabular 데이터셋(분류 253, 회귀 97)으로 사전학습한 뒤 다운스트림별 파인튜닝한다.</t>
-        </is>
-      </c>
-      <c r="G79" s="4" t="inlineStr">
-        <is>
-          <t>사전학습 350개 데이터셋; 평가는 AutoML Multimodal Benchmark·CARTE 벤치마크 등에서 모은 텍스트 특징 포함 50개 데이터셋(데이터셋당 10회 분할, 총 500 런)</t>
-        </is>
-      </c>
-      <c r="H79" s="4" t="inlineStr">
-        <is>
-          <t>CatBoost(tuned), TabM(tuned), TabPFN-v2, CARTE 등 GBDT·tabular DNN·tabular FM</t>
-        </is>
-      </c>
-      <c r="I79" s="4" t="inlineStr">
-        <is>
-          <t>10K 예제 제한/무제한(100K 상한) 두 조건의 분류·회귀 평가, 사전학습 데이터셋 수에 대한 scaling law 분석, head-to-head 승률 분석</t>
-        </is>
-      </c>
-      <c r="J79" s="4" t="inlineStr">
-        <is>
-          <t>AUROC (classification), R2 (regression), normalized score</t>
-        </is>
-      </c>
-      <c r="K79" s="4" t="inlineStr">
-        <is>
-          <t>10K 조건 분류에서 normalized score 0.83으로 TabM-Tuned(0.73), CatBoost-Tuned(0.69), TabPFN-v2(0.67)를 앞섰고, TabPFN-v2 상대 11개 중 8개 데이터셋에서 승리했다. 무제한 조건에서도 0.84로 선두였으며, 사전학습 데이터셋 수에 대한 scaling law가 관찰됐다.</t>
-        </is>
-      </c>
-      <c r="L79" s="4" t="inlineStr">
-        <is>
-          <t>회귀에서는 경쟁력은 있으나 GBDT가 여전히 우세</t>
-        </is>
-      </c>
-      <c r="M79" s="4" t="inlineStr">
-        <is>
-          <t>NeurIPS 2025</t>
-        </is>
-      </c>
-      <c r="N79" s="4" t="n">
-        <v>2025</v>
-      </c>
-      <c r="O79" s="4" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/pdf/2505.18125</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="95" customHeight="1">
-      <c r="A80" s="11" t="inlineStr">
-        <is>
-          <t>CARTE</t>
-        </is>
-      </c>
-      <c r="B80" s="4" t="inlineStr">
-        <is>
-          <t>CARTE: Pretraining and Transfer for Tabular Learning</t>
-        </is>
-      </c>
-      <c r="C80" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/soda-inria/carte</t>
-        </is>
-      </c>
-      <c r="D80" s="4" t="inlineStr">
-        <is>
-          <t>테이블 간 전이는 entity matching·schema matching 같은 데이터 통합 작업을 요구해 왔다. 컬럼 대응 없이도 서로 다른 테이블 간 지식을 전이할 수 있는 구조가 필요하다.</t>
-        </is>
-      </c>
-      <c r="E80" s="4" t="inlineStr">
-        <is>
-          <t>테이블 행을 그래프로 표현해 스키마 매칭 없이 사전학습·전이가 가능한 tabular 신경망(CARTE)을 만드는 것.</t>
-        </is>
-      </c>
-      <c r="F80" s="4" t="inlineStr">
-        <is>
-          <t>각 행을 star graph로 표현하고 셀 값·컬럼명을 문자열 임베딩으로 개방 어휘(open vocabulary) 처리한 뒤, graph-attentional network로 컬럼명·이웃 셀 문맥을 반영한 표현을 학습한다. YAGO3 지식베이스(630만 엔티티, 1,810만 트리플)로 사전학습한 후 다운스트림 테이블에 파인튜닝하며, 매칭되지 않은 컬럼을 가진 테이블 간 공동 학습도 지원한다.</t>
-        </is>
-      </c>
-      <c r="G80" s="4" t="inlineStr">
-        <is>
-          <t>YAGO3 지식그래프(사전학습), Kaggle 등에서 수집한 51개 tabular 데이터셋(회귀 40, 분류 11)</t>
-        </is>
-      </c>
-      <c r="H80" s="4" t="inlineStr">
-        <is>
-          <t>CatBoost·XGBoost 등 트리 모델과 TabPFN을 포함한 42개 베이스라인</t>
-        </is>
-      </c>
-      <c r="I80" s="4" t="inlineStr">
-        <is>
-          <t>샘플 수를 변화시킨 single-table 학습 곡선, 결측치 강건성, 관련 주제 테이블 간 multi-table 전이 실험</t>
-        </is>
-      </c>
-      <c r="J80" s="4" t="inlineStr">
-        <is>
-          <t>AUROC (classification), R2 (regression), normalized score, critical-difference rank</t>
-        </is>
-      </c>
-      <c r="K80" s="4" t="inlineStr">
-        <is>
-          <t>51개 데이터셋에서 42개 베이스라인 대비 평균 순위 1위로 최상의 트리 모델(CatBoost 등)을 능가했고, 특히 고카디널리티 문자열 컬럼이 많은 데이터에서 강했다. 매칭되지 않은 소스 테이블을 추가할수록 중앙값 성능이 오르고 분산이 줄어 cross-table 전이 이득을 입증했다.</t>
-        </is>
-      </c>
-      <c r="L80" s="4" t="inlineStr">
-        <is>
-          <t>명시 없음</t>
-        </is>
-      </c>
       <c r="M80" s="4" t="inlineStr">
         <is>
-          <t>ICML 2024</t>
+          <t>ICLR 2024 (spotlight)</t>
         </is>
       </c>
       <c r="N80" s="4" t="n">
@@ -6389,74 +6378,70 @@
       </c>
       <c r="O80" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2402.16785</t>
+          <t>https://arxiv.org/pdf/2403.01841</t>
         </is>
       </c>
     </row>
     <row r="81" ht="95" customHeight="1">
-      <c r="A81" s="11" t="inlineStr">
-        <is>
-          <t>CM2</t>
+      <c r="A81" s="10" t="inlineStr">
+        <is>
+          <t>UniTabE</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Towards Cross-Table Masked Pretraining for Web Data Mining</t>
-        </is>
-      </c>
-      <c r="C81" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/Chao-Ye/CM2</t>
-        </is>
-      </c>
+          <t>UniTabE: A Universal Pretraining Protocol for Tabular Foundation Model in Data Science</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr"/>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>웹에는 방대한 이질적 테이블이 있으나 기존 tabular 사전학습은 단일 테이블 수준에 머물러 NLP의 'BERT moment'에 해당하는 돌파구가 없었다.</t>
+          <t>NLP의 대규모 사전학습 성공에 비해 tabular 도메인에는 구조가 서로 다른 테이블을 통일적으로 처리하는 범용 사전학습 프로토콜이 없다. 테이블 구조 제약 없이 지식이 태스크·컬럼 변화에 전이되는지가 핵심 질문이다.</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>웹 규모의 이질적 테이블 코퍼스에 대한 masked pretraining으로 범용 tabular 표현을 학습하는 것.</t>
+          <t>테이블 구조에 구애받지 않는 통일된 사전학습 프로토콜로 tabular foundation model을 구축하는 것.</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>이질적 테이블을 통일 인코딩하는 semantic-aware tabular neural network를 설계하고, NLP의 MLM을 테이블에 맞게 변형한 prompt Masked Table Modeling(pMTM) 목적함수로 사전학습한다. OpenML·UCI·Kaggle 등에서 수집한 약 2,000개 테이블·4,600만 샘플 규모의 OpenTabs 코퍼스를 구축해 사용한다.</t>
+          <t>테이블의 기본 요소(컬럼명-값 쌍)를 TabUnit 모듈로 표현한 뒤 Transformer encoder로 정제하고, free-form prompt로 사전학습과 파인튜닝을 통일한다. Kaggle에서 수집한 약 130억(13B) 샘플 규모의 tabular 데이터로 사전학습한다.</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>OpenTabs(약 2,000개 테이블, 4,600만 샘플) 사전학습; 다운스트림 분류 16개, 회귀 6개, 이상탐지·결측치 대체 데이터셋</t>
+          <t>Kaggle 기반 대규모 사전학습 코퍼스(약 13B 샘플), 다수의 분류·회귀 벤치마크 데이터셋</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr">
         <is>
-          <t>FT-Transformer 등 tabular 딥러닝, 트리 계열, 기존 tabular 사전학습 방법</t>
+          <t>기존 tabular 딥러닝 및 트리 계열 베이스라인</t>
         </is>
       </c>
       <c r="I81" s="4" t="inlineStr">
         <is>
-          <t>supervised 파인튜닝, few-shot(5-shot 등), 이상탐지·결측 대체 등 다양한 다운스트림 전이 실험</t>
+          <t>분류·회귀 다운스트림 전이, 태스크 간 일반화·전이성, 시간에 따른 컬럼 증가(incremental columns) 적응 실험</t>
         </is>
       </c>
       <c r="J81" s="4" t="inlineStr">
         <is>
-          <t>AUC (classification), RMSE (regression), F1 (anomaly detection)</t>
+          <t>AUC (classification), RMSE/R2 (regression)</t>
         </is>
       </c>
       <c r="K81" s="4" t="inlineStr">
         <is>
-          <t>16개 분류 데이터셋 중 12개에서 모든 베이스라인을 상회하며 SOTA 평균 성능을 달성했고, few-shot(특히 5-shot)에서 from-scratch 대비 사전학습 이득이 가장 컸다. 기존 연구가 10~52개 테이블로 사전학습한 데 비해 약 2,000개 테이블로 규모를 확장했다.</t>
+          <t>약 13B 샘플의 Kaggle 사전학습으로 다수 벤치마크의 분류·회귀 태스크에서 베이스라인 대비 우수한 성능을 보였고, 구조가 다른 테이블·증분 컬럼 시나리오에도 적응 가능함을 보였다.</t>
         </is>
       </c>
       <c r="L81" s="4" t="inlineStr">
         <is>
-          <t>명시 없음</t>
+          <t>명시 없음 (공식 코드 저장소 미확인)</t>
         </is>
       </c>
       <c r="M81" s="4" t="inlineStr">
         <is>
-          <t>WWW 2024</t>
+          <t>ICLR 2024</t>
         </is>
       </c>
       <c r="N81" s="4" t="n">
@@ -6464,281 +6449,281 @@
       </c>
       <c r="O81" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2307.04308</t>
+          <t>https://arxiv.org/pdf/2307.09249</t>
         </is>
       </c>
     </row>
     <row r="82" ht="95" customHeight="1">
-      <c r="A82" s="11" t="inlineStr">
-        <is>
-          <t>GTL</t>
+      <c r="A82" s="10" t="inlineStr">
+        <is>
+          <t>TabLLM</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>From Supervised to Generative: A Novel Paradigm for Tabular Deep Learning with Large Language Models</t>
+          <t>TabLLM: Few-shot Classification of Tabular Data with Large Language Models</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/microsoft/Industrial-Foundation-Models</t>
+          <t>https://github.com/clinicalml/TabLLM</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>기존 tabular 딥러닝은 지식 전이, 소수 데이터 일반화, 지시 따르기 등 범용 모델 요구를 충족하지 못한다. LLM의 zero-shot 일반화와 in-context learning을 tabular 예측에 이식하려 한다.</t>
+          <t>라벨이 극히 적은 tabular 분류에서 딥러닝은 GBDT에 밀려 왔으나, LLM에 내재된 세계 지식(사전 지식)을 활용하면 zero/few-shot 예측이 가능할 수 있다.</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>다양한 tabular 데이터에 대한 생성적 continued pretraining(GTL)으로 LLM에 범용 tabular 예측 능력을 부여하는 것.</t>
+          <t>테이블 행을 자연어로 직렬화해 LLM으로 zero-shot·few-shot tabular 분류를 수행하는 것.</t>
         </is>
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>테이블을 지시·특징·타깃이 포함된 텍스트 템플릿으로 변환해 LLaMA-2를 384개 공개 데이터셋 위에서 생성적(next-token) 방식으로 continued pretraining한다. 프롬프트 기반 zero-shot과 in-context 예시를 통한 few-shot 예측을 하나의 생성 패러다임으로 통일하고, 수렴·스케일링 거동과 데이터 템플릿 영향을 분석한다.</t>
+          <t>테이블 행을 템플릿, table-to-text 모델, LLM 등 여러 직렬화 방식으로 자연어 문자열로 변환하고 태스크 설명과 함께 LLM(T0 계열)에 프롬프트한다. few-shot 설정에서는 소수 라벨 예시로 LLM을 파라미터 효율적으로(t-few) 파인튜닝한다.</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>384개 공개 tabular 데이터셋(분류·회귀)</t>
+          <t>심장질환, 소득 예측, 신용 분류 등 9개 공개 tabular 데이터셋(+비공개 의료 데이터셋)</t>
         </is>
       </c>
       <c r="H82" s="4" t="inlineStr">
         <is>
-          <t>전통적 지도학습 tabular 방법들과 GPT-4 등 범용 LLM</t>
+          <t>GBDT(XGBoost 등) 전통 베이스라인과 기존 tabular 딥러닝 방법, 직렬화 방식 간 상호 비교</t>
         </is>
       </c>
       <c r="I82" s="4" t="inlineStr">
         <is>
-          <t>zero-shot·in-context learning 평가, 스케일링/수렴 분석, 데이터 템플릿 ablation</t>
+          <t>shot 수(0~다수)를 변화시키며 성능 곡선 비교, 직렬화 방식 ablation</t>
         </is>
       </c>
       <c r="J82" s="4" t="inlineStr">
         <is>
-          <t>zero-shot / in-context accuracy (classification), regression error</t>
+          <t>AUC (zero-shot / few-shot classification)</t>
         </is>
       </c>
       <c r="K82" s="4" t="inlineStr">
         <is>
-          <t>GTL로 강화된 LLaMA-2는 384개 데이터셋 실험에서 파인튜닝 없이 zero-shot·ICL 성능이 전통 방법을 능가했고, 일부 태스크에서는 GPT-4에 필적했다.</t>
+          <t>9개 공개 벤치마크에서 기존 tabular 딥러닝 분류 방법을 능가했고, zero-shot에서도 대부분 non-trivial한 성능을 얻어 LLM의 사전 지식 활용을 입증했다. 특히 very-few-shot 구간에서 GBDT 등 강한 전통 베이스라인과 경쟁하거나 능가했다.</t>
         </is>
       </c>
       <c r="L82" s="4" t="inlineStr">
         <is>
-          <t>명시 없음</t>
+          <t>명시 없음 (비공개 의료 데이터 부분은 코드 미공개)</t>
         </is>
       </c>
       <c r="M82" s="4" t="inlineStr">
         <is>
-          <t>KDD 2024</t>
+          <t>AISTATS 2023</t>
         </is>
       </c>
       <c r="N82" s="4" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="O82" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2310.07338</t>
+          <t>https://arxiv.org/pdf/2210.10723</t>
         </is>
       </c>
     </row>
     <row r="83" ht="95" customHeight="1">
-      <c r="A83" s="11" t="inlineStr">
-        <is>
-          <t>LLM-TabSurvey</t>
+      <c r="A83" s="10" t="inlineStr">
+        <is>
+          <t>XTab</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Large Language Models(LLMs) on Tabular Data: Prediction, Generation, and Understanding -- A Survey</t>
-        </is>
-      </c>
-      <c r="C83" s="4" t="inlineStr"/>
+          <t>XTab: Cross-table Pretraining for Tabular Transformers</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/BingzhaoZhu/XTab</t>
+        </is>
+      </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>LLM을 tabular 예측·생성·이해에 적용하는 연구가 급증했으나 핵심 기법·메트릭·데이터셋·미해결 과제를 아우르는 종합 정리가 없었다.</t>
+          <t>기존 tabular self-supervised 학습은 단일 테이블에 갇혀 여러 테이블 간 정보를 활용하지 못하고 새로운 테이블로 일반화되지 않는다. 테이블마다 컬럼 타입·개수가 달라 교차 테이블 사전학습이 어렵다는 문제를 겨냥한다.</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>tabular 데이터에 대한 LLM 활용(예측·생성·이해)을 체계적으로 분류·정리하는 것.</t>
+          <t>도메인이 다른 다수의 테이블로 tabular transformer를 사전학습하는 범용 cross-table pretraining 프레임워크를 만드는 것.</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>LLM 기반 tabular 모델링을 예측(prediction), 데이터 생성(generation), 이해(table QA·comprehension)의 3개 축으로 나눠 직렬화·프롬프트·파인튜닝 등 기법을 분류한다. 각 축의 데이터셋·메트릭 분류체계를 제공하고 연구 공백과 향후 방향을 제시한다.</t>
+          <t>테이블별 독립 featurizer로 이질적 스키마를 흡수하고, 공유 백본(transformer)은 federated learning 방식으로 다수 테이블에 걸쳐 사전학습한다. 사전학습된 공유 가중치를 초기값으로 FT-Transformer 등 다양한 tabular transformer를 다운스트림 테이블에 파인튜닝한다.</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr">
         <is>
-          <t>해당 없음 (서베이; 각 축별 공개 데이터셋·벤치마크 분류 제공)</t>
+          <t>OpenML-AutoML Benchmark(AMLB)의 84개 tabular 예측 태스크(회귀·이진·다중 분류)</t>
         </is>
       </c>
       <c r="H83" s="4" t="inlineStr">
         <is>
-          <t>해당 없음 (기존 방법론 간 정성적 비교·분류)</t>
+          <t>무(無)사전학습 tabular transformer(FT-Transformer 등)와 기존 SOTA tabular 딥러닝 모델, 트리 기반 AutoML 베이스라인</t>
         </is>
       </c>
       <c r="I83" s="4" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>사전학습 유무·사전학습 스텝 수(0/1k/2k)에 따른 다운스트림 파인튜닝 성능 비교, 회귀/이진/다중 분류 전반의 순위 비교</t>
         </is>
       </c>
       <c r="J83" s="4" t="inlineStr">
         <is>
-          <t>N/A (survey)</t>
+          <t>ROC-AUC (binary), RMSE (regression), average rank on AMLB tasks</t>
         </is>
       </c>
       <c r="K83" s="4" t="inlineStr">
         <is>
-          <t>41페이지, 8개 표 분량으로 LLM 기반 tabular 예측·생성·이해 기법과 데이터셋·메트릭의 분류체계를 정리했고, 직렬화 방식·파인튜닝 전략별 장단점과 미해결 과제(수치 표현, 대규모 테이블 처리 등)를 도출했다. TabLLM·GTL류 LLM 기반 예측 계열의 표준 참조 서베이로 자리잡았다.</t>
+          <t>84개 AMLB 태스크에서 여러 tabular transformer의 일반화 성능·학습 속도·최종 성능을 일관되게 향상시켰고, XTab으로 사전학습한 FT-Transformer는 회귀·이진·다중 분류에서 타 tabular 딥러닝 SOTA보다 우수했다. 사전학습 스텝(0→2000)이 늘수록 다운스트림 성능이 개선되는 경향을 보였다.</t>
         </is>
       </c>
       <c r="L83" s="4" t="inlineStr">
         <is>
-          <t>빠르게 발전하는 분야 특성상 2024년 이후 모델은 미포함</t>
+          <t>명시 없음 (재현에는 AWS 분산 학습 인프라가 필요하다고 저장소에 기술)</t>
         </is>
       </c>
       <c r="M83" s="4" t="inlineStr">
         <is>
-          <t>TMLR 2024</t>
+          <t>ICML 2023</t>
         </is>
       </c>
       <c r="N83" s="4" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="O83" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2402.17944</t>
+          <t>https://arxiv.org/pdf/2305.06090</t>
         </is>
       </c>
     </row>
     <row r="84" ht="95" customHeight="1">
       <c r="A84" s="11" t="inlineStr">
         <is>
-          <t>LTM-Position</t>
+          <t>BAPS</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Why Tabular Foundation Models Should Be a Research Priority</t>
+          <t>Balanced Adaptive Prototype Selection for Scalable TabPFN Inference on Large-Scale Tabular Data</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr"/>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>텍스트·이미지 foundation model에 연구 자원이 쏠리는 동안 여러 분야의 지배적 데이터 양식인 tabular 데이터는 규모·역량 면에서 크게 뒤처져 있다.</t>
+          <t>사전학습된 표 형식 파운데이션 모델은 강력하지만 제한된 추론 문맥 길이 때문에 대규모 데이터셋 적용이 어렵다.</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>Large Tabular Model(LTM) 개발을 ML 커뮤니티의 우선 연구 과제로 제안하는 것.</t>
+          <t>모델 수정·재학습 없이 정보 보존형 압축 문맥을 구성하여 TabPFN을 백만 행 규모 데이터로 확장한다.</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>포지션 논문으로서 tabular 도메인의 연구 공백을 진단하고 LTM 개념을 정의한다. few-shot tabular 모델, 데이터 사이언스 자동화, OOD 합성 데이터, 다학제 과학 발견 등 LTM의 파급 효과와 연구 로드맵(데이터, 아키텍처, 평가 과제)을 논한다.</t>
+          <t>Balanced Adaptive Prototype Selection(BAPS)은 대표 구조, 결정 경계 정보, 국소 밀도, 클래스 균형, 특징 공간 다양성을 동시에 보존하는 프로토타입 선택으로 압축 문맥을 만든다. 사전학습 모델을 전혀 수정하지 않는 순수 문맥 구성 접근이다.</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>해당 없음 (포지션 논문)</t>
+          <t>백만 행 규모의 HIGGS, SUSY 데이터셋</t>
         </is>
       </c>
       <c r="H84" s="4" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>전체 데이터 문맥 및 기존 문맥 선택 방식 대비 예측 성능·캘리브레이션</t>
         </is>
       </c>
       <c r="I84" s="4" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>512 프로토타입으로 압축한 문맥에서의 예측·캘리브레이션 평가, GPU 없이 Intel Core i7 CPU와 16GB RAM만으로 수행</t>
         </is>
       </c>
       <c r="J84" s="4" t="inlineStr">
         <is>
-          <t>N/A (position paper)</t>
+          <t>predictive accuracy, calibration reliability, context compression ratio</t>
         </is>
       </c>
       <c r="K84" s="4" t="inlineStr">
         <is>
-          <t>tabular 데이터가 다수 분야의 지배적 양식임에도 연구 관심이 미미함을 지적하고, 단일 데이터셋 고립 분석에서 관련 데이터셋 맥락화로의 전환을 LTM의 핵심 가치로 제시했다. TabPFN류 초기 시도를 넘어서는 스케일업 필요성을 논증해 이후 tabular FM 연구의 방향 설정에 널리 인용된다.</t>
+          <t>512개 프로토타입만으로 약 1,953배의 문맥 압축을 달성하면서 강한 예측 성능과 신뢰할 만한 캘리브레이션을 유지했고, GPU 없는 일반 CPU 환경에서 백만 행 데이터에 TabPFN을 적용할 수 있음을 보였다.</t>
         </is>
       </c>
       <c r="L84" s="4" t="inlineStr">
         <is>
-          <t>실험적 검증이 없는 포지션 논문</t>
+          <t>명시 없음</t>
         </is>
       </c>
       <c r="M84" s="4" t="inlineStr">
         <is>
-          <t>ICML 2024 (position paper)</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="N84" s="4" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="O84" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2405.01147</t>
+          <t>https://arxiv.org/pdf/2608.12989</t>
         </is>
       </c>
     </row>
     <row r="85" ht="95" customHeight="1">
       <c r="A85" s="11" t="inlineStr">
         <is>
-          <t>TabuLa-8B</t>
+          <t>ClusterAttn</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Large Scale Transfer Learning for Tabular Data via Language Modeling</t>
-        </is>
-      </c>
-      <c r="C85" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/mlfoundations/rtfm</t>
-        </is>
-      </c>
+          <t>ClusterAttention: A training-free speedup of bidirectional attention</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr"/>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>언어·비전에서 foundation model이 태스크별 모델 개발을 대체했지만 tabular 도메인에는 그런 전이학습 패러다임이 부재하다. 웹 규모 테이블 코퍼스로 LLM을 학습하면 보지 못한 테이블에 대한 zero/few-shot 예측이 가능한지 검증한다.</t>
+          <t>TabPFN류 모델의 양방향 어텐션은 대규모 문맥에서 연산 병목이 되지만, 기존 희소 어텐션 가속 기법은 재학습이나 오프라인 캘리브레이션을 요구하거나 단일 패스 비정형 입력에 적용되지 못했다.</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>TabLib 코퍼스로 파인튜닝한 LLM(TabuLa-8B)으로 대규모 tabular 전이학습(zero/few-shot 예측)을 실현하는 것.</t>
+          <t>재학습 없이 양방향 어텐션을 블록 희소화하여 TabPFN-3 추론을 가속한다.</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>TabLib에서 필터링·품질 관리를 거쳐 400만여 개 테이블·21억 행의 학습 데이터(T4)를 추출하고, Llama 3-8B를 tabular 예측(분류·구간화 회귀)용으로 파인튜닝한다. 행 단위 예측에 맞춘 novel packing·attention 마스킹 기법을 도입한다.</t>
+          <t>각 어텐션 헤드의 key-query 기하에 적응하는 고속 재귀 클러스터링으로 블록 희소 어텐션을 구성하며, 클러스터 크기를 2의 거듭제곱으로 설정해 GPU에서 밀집 어텐션과 동일한 상호작용당 지연시간을 얻는다. 희소 어텐션 출력 오차의 해석적 표현을 유도해 조밀한 클러스터가 오히려 큰 오차를 낼 수 있음을 설명하고, 센트로이드 보상(centroid compensation)으로 이를 상쇄한다.</t>
         </is>
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
-          <t>TabLib 유래 T4 코퍼스(2.1B 행, 4M+ 테이블) 학습; 329개 데이터셋 평가 스위트</t>
+          <t>대규모 표 형식 데이터(TabPFN-3 추론), 비디오 생성(Wan 2.1-14B T2V)</t>
         </is>
       </c>
       <c r="H85" s="4" t="inlineStr">
         <is>
-          <t>XGBoost, TabPFN 등 SOTA tabular 예측 모델(타깃 데이터로 명시적으로 학습된 조건 포함)</t>
+          <t>밀집(dense) 어텐션, 선도적 어텐션 가속 기법들</t>
         </is>
       </c>
       <c r="I85" s="4" t="inlineStr">
         <is>
-          <t>미학습 테이블에 대한 zero-shot 예측, 1~32 shot few-shot(타깃 파인튜닝 없음) 비교, 상대 모델에 최대 16배 데이터를 준 조건 비교</t>
+          <t>TabPFN-3 추론 가속 대 정확도 유지율 측정, 비디오 생성에서 기존 가속 기법과 출력 충실도-속도 비교</t>
         </is>
       </c>
       <c r="J85" s="4" t="inlineStr">
         <is>
-          <t>zero-shot / few-shot accuracy (percentage points vs. random and baselines)</t>
+          <t>speedup factor, retained accuracy vs dense attention, output error</t>
         </is>
       </c>
       <c r="K85" s="4" t="inlineStr">
         <is>
-          <t>329개 데이터셋에서 zero-shot 정확도가 무작위 추측보다 15pp 이상 높았는데 이는 XGBoost·TabPFN 등 기존 모델로는 불가능한 능력이다. 1~32 shot에서는 동량 또는 최대 16배 많은 데이터로 학습된 XGBoost·TabPFN보다 5~15pp 더 정확했다.</t>
+          <t>TabPFN-3를 2~6배 가속하면서 밀집 어텐션 정확도의 99% 이상을 유지했으며, 단일 패스 비정형 입력에 성공적으로 적용된 최초의 training-free 어텐션 가속 기법이다. 비디오 생성에서도 기존 선도 기법보다 더 큰 가속으로 밀집 어텐션에 더 가까운 출력을 냈다.</t>
         </is>
       </c>
       <c r="L85" s="4" t="inlineStr">
@@ -6748,364 +6733,360 @@
       </c>
       <c r="M85" s="4" t="inlineStr">
         <is>
-          <t>NeurIPS 2024</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="N85" s="4" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="O85" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2406.12031</t>
+          <t>https://arxiv.org/pdf/2608.26965</t>
         </is>
       </c>
     </row>
     <row r="86" ht="95" customHeight="1">
       <c r="A86" s="11" t="inlineStr">
         <is>
-          <t>TP-BERTa</t>
+          <t>EnterpriseTab</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Making Pre-trained Language Models Great on Tabular Prediction</t>
-        </is>
-      </c>
-      <c r="C86" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/jyansir/tp-berta</t>
-        </is>
-      </c>
+          <t>Exploring Differences Between Tabular Enterprise Data and Public Benchmarks</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr"/>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>이미지·언어에서 확립된 전이학습이 tabular 예측에서는 미활용 상태이며, LM을 그대로 쓰면 수치 특징 값을 제대로 표현하지 못한다. 수치값의 크기 정보를 LM 토큰 공간에 이식하는 것이 관건이다.</t>
+          <t>표 형식 모델과 벤치마크가 급증했지만 기업(enterprise) 데이터의 특성은 거의 연구되지 않았으며, 공개 벤치마크 성능이 실제 업무 데이터로 이어지는지 불분명하다.</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>수치 특징을 다룰 수 있게 특화 사전학습한 언어 모델(TP-BERTa)로 tabular 예측에서 GBDT급 성능을 내는 것.</t>
+          <t>기업 표 형식 데이터의 통계적 특성을 분석하고 공개 벤치마크와의 성능 괴리를 실증한다.</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>수치값을 상대적 크기 기반 이산 토큰으로 바꾸는 relative magnitude tokenization(RMT)으로 수치를 LM 어휘에 통합한다. intra-feature attention(IFA)으로 특징명과 값을 결합해 특징 단위 표현을 만들고, RoBERTa를 101개 이진 분류 + 101개 회귀 데이터셋(약 1천만 샘플)으로 사전학습한다.</t>
+          <t>기업 데이터의 데이터 통계량을 공개 표 형식 벤치마크와 비교 분석하고, TabPFN·TabICL·ConTextTab 같은 표 형식 모델들의 성능을 양쪽에서 측정하여 일반화 여부를 검증한다.</t>
         </is>
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>사전학습 202개 데이터셋(약 10M 샘플), 다운스트림 145개 데이터셋(이진 분류 80개, 회귀 65개)</t>
+          <t>실제 기업(enterprise) 표 형식 데이터와 공개 표 형식 벤치마크</t>
         </is>
       </c>
       <c r="H86" s="4" t="inlineStr">
         <is>
-          <t>tuned XGBoost/CatBoost 등 GBDT, FT-Transformer 등 tabular DNN, 기존 LM 기반 tabular 접근</t>
+          <t>TabPFN, TabICL, ConTextTab 등 표 형식 파운데이션 모델 간 및 데이터 소스 간 성능 비교</t>
         </is>
       </c>
       <c r="I86" s="4" t="inlineStr">
         <is>
-          <t>default/tuned 설정별 평균 순위 비교, 범주형 특징 비중에 따른 성능 분석, RMT/IFA ablation</t>
+          <t>데이터 통계 특성 비교 분석, 동일 모델의 벤치마크 대 기업 데이터 성능 교차 측정</t>
         </is>
       </c>
       <c r="J86" s="4" t="inlineStr">
         <is>
-          <t>AUC (binary classification), RMSE (regression), average rank</t>
+          <t>data statistics, model performance measurements across benchmark vs enterprise data</t>
         </is>
       </c>
       <c r="K86" s="4" t="inlineStr">
         <is>
-          <t>145개 다운스트림에서 default 설정 기준 평균 순위 5.8로 tuned XGBoost(6.2), tuned CatBoost(5.9)와 대등한 GBDT급 성능을 달성했다. 범주형 특징이 우세한 데이터셋에서는 순위 4.4로 tuned CatBoost(7.1)를 크게 앞섰고, RMT 인코딩은 기존 LM 인코딩 대비 AUC를 최대 12.45% 개선했다.</t>
+          <t>기업 데이터는 공개 벤치마크와 뚜렷이 다르며, 전형적 벤치마크에서 잘하는 모델이 실제 기업 데이터에서 저조할 수 있고 그 역도 성립함을 보였다. 이는 기업급 특성을 가진 추가 벤치마크의 필요성을 시사한다.</t>
         </is>
       </c>
       <c r="L86" s="4" t="inlineStr">
         <is>
-          <t>명시 없음</t>
+          <t>기업 데이터의 비공개 특성상 재현 가능한 공개 벤치마크 제공에는 한계가 있다.</t>
         </is>
       </c>
       <c r="M86" s="4" t="inlineStr">
         <is>
-          <t>ICLR 2024 (spotlight)</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="N86" s="4" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="O86" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2403.01841</t>
+          <t>https://arxiv.org/pdf/2606.30452</t>
         </is>
       </c>
     </row>
     <row r="87" ht="95" customHeight="1">
       <c r="A87" s="11" t="inlineStr">
         <is>
-          <t>UniTabE</t>
+          <t>GOTabPFN</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>UniTabE: A Universal Pretraining Protocol for Tabular Foundation Model in Data Science</t>
-        </is>
-      </c>
-      <c r="C87" s="4" t="inlineStr"/>
+          <t>GOTabPFN: From Feature Ordering to Compact Tokenization for Tabular Foundation Models on High-Dimensional Data</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/zadid6pretam/GOTabPFN</t>
+        </is>
+      </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>NLP의 대규모 사전학습 성공에 비해 tabular 도메인에는 구조가 서로 다른 테이블을 통일적으로 처리하는 범용 사전학습 프로토콜이 없다. 테이블 구조 제약 없이 지식이 태스크·컬럼 변화에 전이되는지가 핵심 질문이다.</t>
+          <t>소형 표 형식 파운데이션 모델은 토큰 예산 제약 때문에 고차원-저표본(HDLSS) 데이터에서 성능이 불안정하며, 대형 백본 재학습 없이 이를 해결할 방법이 필요하다.</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>테이블 구조에 구애받지 않는 통일된 사전학습 프로토콜로 tabular foundation model을 구축하는 것.</t>
+          <t>특징 순서 최적화와 압축 토크나이제이션으로 재학습 없이 TabPFN류 모델을 고차원 데이터에 적용 가능하게 만든다.</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>테이블의 기본 요소(컬럼명-값 쌍)를 TabUnit 모듈로 표현한 뒤 Transformer encoder로 정제하고, free-form prompt로 사전학습과 파인튜닝을 통일한다. Kaggle에서 수집한 약 130억(13B) 샘플 규모의 tabular 데이터로 사전학습한다.</t>
+          <t>Graph-guided Ordering with Local Refinement(GO-LR)로 특징 순서를 최적화하며 이것이 가중 Minimum Linear Arrangement 문제와 동치임을 보인다. 이어 Neuro-Inspired Subunit Compression(NSC) 유닛이 국소적으로 인접한 정렬 특징들을 메타 특징으로 풀링하여 HDLSS 체제에 맞는 압축 표현을 만든다.</t>
         </is>
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>Kaggle 기반 대규모 사전학습 코퍼스(약 13B 샘플), 다수의 분류·회귀 벤치마크 데이터셋</t>
+          <t>고차원-저표본(HDLSS) 특성의 표 형식 벤치마크들</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr">
         <is>
-          <t>기존 tabular 딥러닝 및 트리 계열 베이스라인</t>
+          <t>특징 순서/압축을 적용하지 않은 TabPFN류 기본 모델 및 표 형식 베이스라인</t>
         </is>
       </c>
       <c r="I87" s="4" t="inlineStr">
         <is>
-          <t>분류·회귀 다운스트림 전이, 태스크 간 일반화·전이성, 시간에 따른 컬럼 증가(incremental columns) 적응 실험</t>
+          <t>타이트한 토큰 예산 하에서의 안정성·정확도 평가, 순서화-압축 구성요소 검증</t>
         </is>
       </c>
       <c r="J87" s="4" t="inlineStr">
         <is>
-          <t>AUC (classification), RMSE/R2 (regression)</t>
+          <t>accuracy, stability under tight token budgets</t>
         </is>
       </c>
       <c r="K87" s="4" t="inlineStr">
         <is>
-          <t>약 13B 샘플의 Kaggle 사전학습으로 다수 벤치마크의 분류·회귀 태스크에서 베이스라인 대비 우수한 성능을 보였고, 구조가 다른 테이블·증분 컬럼 시나리오에도 적응 가능함을 보였다.</t>
+          <t>GOTabPFN이 타이트한 토큰 예산 조건에서 안정성과 정확도를 모두 개선하여, 백본 재학습 없이 소형 표 형식 파운데이션 모델을 고차원 데이터에 효과적으로 확장할 수 있음을 보였다.</t>
         </is>
       </c>
       <c r="L87" s="4" t="inlineStr">
         <is>
-          <t>명시 없음 (공식 코드 저장소 미확인)</t>
+          <t>명시 없음</t>
         </is>
       </c>
       <c r="M87" s="4" t="inlineStr">
         <is>
-          <t>ICLR 2024</t>
+          <t>ICML 2026</t>
         </is>
       </c>
       <c r="N87" s="4" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="O87" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2307.09249</t>
+          <t>https://arxiv.org/pdf/2606.05441</t>
         </is>
       </c>
     </row>
     <row r="88" ht="95" customHeight="1">
       <c r="A88" s="11" t="inlineStr">
         <is>
-          <t>TabLLM</t>
+          <t>LimiX-2M</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>TabLLM: Few-shot Classification of Tabular Data with Large Language Models</t>
+          <t>LimiX-2M: Mitigating Low-Rank Collapse and Attention Bottlenecks in Tabular Foundation Models</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/clinicalml/TabLLM</t>
+          <t>https://github.com/limix-ldm-ai/LimiX</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>라벨이 극히 적은 tabular 분류에서 딥러닝은 GBDT에 밀려 왔으나, LLM에 내재된 세계 지식(사전 지식)을 활용하면 zero/few-shot 예측이 가능할 수 있다.</t>
+          <t>표 형식 파운데이션 모델이 트리 앙상블에 필적하지만, 표준적인 affine 스칼라 토크나이제이션은 저층 표현의 저랭크 붕괴(low-rank collapse)와 어텐션 병목을 일으켜 연산 효율이 낮다.</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>테이블 행을 자연어로 직렬화해 LLM으로 zero-shot·few-shot tabular 분류를 수행하는 것.</t>
+          <t>값 인지 토크나이제이션과 계산 재배열로 소형 모델의 정확도-효율 트레이드오프를 개선한다.</t>
         </is>
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>테이블 행을 템플릿, table-to-text 모델, LLM 등 여러 직렬화 방식으로 자연어 문자열로 변환하고 태스크 설명과 함께 LLM(T0 계열)에 프롬프트한다. few-shot 설정에서는 소수 라벨 예시로 LLM을 파라미터 효율적으로(t-few) 파인튜닝한다.</t>
+          <t>통합 tokenize-and-route 프레임워크를 제안한다. RaBEL이 각 스칼라 값을 국소화된 RBF 특징으로 확장해 조건화와 얕은 층의 유효 랭크를 개선하고, 양방향 블록을 S→N→F 순서로 재배열해 계산을 readout에 정렬시킨다.</t>
         </is>
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
-          <t>심장질환, 소득 예측, 신용 분류 등 9개 공개 tabular 데이터셋(+비공개 의료 데이터셋)</t>
+          <t>널리 쓰이는 표 형식 벤치마크들</t>
         </is>
       </c>
       <c r="H88" s="4" t="inlineStr">
         <is>
-          <t>GBDT(XGBoost 등) 전통 베이스라인과 기존 tabular 딥러닝 방법, 직렬화 방식 간 상호 비교</t>
+          <t>더 큰 규모의 TabPFN-v2, TabICL</t>
         </is>
       </c>
       <c r="I88" s="4" t="inlineStr">
         <is>
-          <t>shot 수(0~다수)를 변화시키며 성능 곡선 비교, 직렬화 방식 ablation</t>
+          <t>벤치마크 정확도 비교와 학습·추론 비용 분석, 토크나이제이션·블록 순서 설계 검증</t>
         </is>
       </c>
       <c r="J88" s="4" t="inlineStr">
         <is>
-          <t>AUC (zero-shot / few-shot classification)</t>
+          <t>benchmark accuracy/rank, training and inference cost, effective rank</t>
         </is>
       </c>
       <c r="K88" s="4" t="inlineStr">
         <is>
-          <t>9개 공개 벤치마크에서 기존 tabular 딥러닝 분류 방법을 능가했고, zero-shot에서도 대부분 non-trivial한 성능을 얻어 LLM의 사전 지식 활용을 입증했다. 특히 very-few-shot 구간에서 GBDT 등 강한 전통 베이스라인과 경쟁하거나 능가했다.</t>
+          <t>단 2M 파라미터의 LimiX-2M이 자신보다 큰 TabPFN-v2와 TabICL을 표 형식 벤치마크에서 상회하면서 학습·추론 비용을 동시에 절감했다.</t>
         </is>
       </c>
       <c r="L88" s="4" t="inlineStr">
         <is>
-          <t>명시 없음 (비공개 의료 데이터 부분은 코드 미공개)</t>
+          <t>명시 없음</t>
         </is>
       </c>
       <c r="M88" s="4" t="inlineStr">
         <is>
-          <t>AISTATS 2023</t>
+          <t>ICML 2026</t>
         </is>
       </c>
       <c r="N88" s="4" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="O88" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2210.10723</t>
+          <t>https://arxiv.org/pdf/2606.04485</t>
         </is>
       </c>
     </row>
     <row r="89" ht="95" customHeight="1">
       <c r="A89" s="11" t="inlineStr">
         <is>
-          <t>XTab</t>
+          <t>SpurRoute</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>XTab: Cross-table Pretraining for Tabular Transformers</t>
-        </is>
-      </c>
-      <c r="C89" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/BingzhaoZhu/XTab</t>
-        </is>
-      </c>
+          <t>Entangled by Design: Spurious Intra-Variable Signal Routing in Tabular In-Context Learners</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr"/>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>기존 tabular self-supervised 학습은 단일 테이블에 갇혀 여러 테이블 간 정보를 활용하지 못하고 새로운 테이블로 일반화되지 않는다. 테이블마다 컬럼 타입·개수가 달라 교차 테이블 사전학습이 어렵다는 문제를 겨냥한다.</t>
+          <t>하나의 특징이 진짜 인과 신호와 장비 아티팩트 같은 허위 신호를 함께 담고 있을 때(예: 병원별 측정 장비 편향), 인컨텍스트 학습기는 허위 신호를 통해 예측을 라우팅하여 새 환경에서 조용히 실패할 수 있다.</t>
         </is>
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>도메인이 다른 다수의 테이블로 tabular transformer를 사전학습하는 범용 cross-table pretraining 프레임워크를 만드는 것.</t>
+          <t>표 형식 인컨텍스트 학습기의 변수 내 허위 신호 라우팅을 이론적으로 정식화하고 경량 완화책을 제시한다.</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>테이블별 독립 featurizer로 이질적 스키마를 흡수하고, 공유 백본(transformer)은 federated learning 방식으로 다수 테이블에 걸쳐 사전학습한다. 사전학습된 공유 가중치를 초기값으로 FT-Transformer 등 다양한 tabular transformer를 다운스트림 테이블에 파인튜닝한다.</t>
+          <t>X=[C; αS; η] 형태의 복합 표현에서 ridge ICL이 문맥 크기와 무관하게 허위 라우팅을 피할 수 없음을 증명하고, CSR ∝ ρ_S/ρ_C의 닫힌 형식 특성화를 유도한다. 약한 환경 라벨만 요구하는 두 가지 완화책(환경 층화 문맥 구성, S-swap 증강)을 제안한다.</t>
         </is>
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>OpenML-AutoML Benchmark(AMLB)의 84개 tabular 예측 태스크(회귀·이진·다중 분류)</t>
+          <t>인과/허위 신호 부분공간을 통제한 합성 복합 표현 데이터</t>
         </is>
       </c>
       <c r="H89" s="4" t="inlineStr">
         <is>
-          <t>무(無)사전학습 tabular transformer(FT-Transformer 등)와 기존 SOTA tabular 딥러닝 모델, 트리 기반 AutoML 베이스라인</t>
+          <t>선형(ridge) ICL 이론 예측 vs TabPFN의 실증 거동</t>
         </is>
       </c>
       <c r="I89" s="4" t="inlineStr">
         <is>
-          <t>사전학습 유무·사전학습 스텝 수(0/1k/2k)에 따른 다운스트림 파인튜닝 성능 비교, 회귀/이진/다중 분류 전반의 순위 비교</t>
+          <t>닫힌 형식 예측의 실증 검증, 문맥 크기에 따른 허위 라우팅 증폭 측정, 완화책 적용 전후 CSR 비교</t>
         </is>
       </c>
       <c r="J89" s="4" t="inlineStr">
         <is>
-          <t>ROC-AUC (binary), RMSE (regression), average rank on AMLB tasks</t>
+          <t>Causal-Spurious Routing ratio (CSR), correlation with closed-form prediction, causal sensitivity</t>
         </is>
       </c>
       <c r="K89" s="4" t="inlineStr">
         <is>
-          <t>84개 AMLB 태스크에서 여러 tabular transformer의 일반화 성능·학습 속도·최종 성능을 일관되게 향상시켰고, XTab으로 사전학습한 FT-Transformer는 회귀·이진·다중 분류에서 타 tabular 딥러닝 SOTA보다 우수했다. 사전학습 스텝(0→2000)이 늘수록 다운스트림 성능이 개선되는 경향을 보였다.</t>
+          <t>닫힌 형식 특성화가 선형 ICL에서 r=0.997, TabPFN에서 r=0.979로 확인되었고, 직관과 달리 문맥이 클수록 허위 라우팅이 최대 1.74배 증폭되었다. S-swap 증강은 허위 라우팅을 선형 ICL에서 74%, TabPFN에서 98.8% 줄이면서 TabPFN의 인과 민감도를 8.4배 높였다.</t>
         </is>
       </c>
       <c r="L89" s="4" t="inlineStr">
         <is>
-          <t>명시 없음 (재현에는 AWS 분산 학습 인프라가 필요하다고 저장소에 기술)</t>
+          <t>명시 없음</t>
         </is>
       </c>
       <c r="M89" s="4" t="inlineStr">
         <is>
-          <t>ICML 2023</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="N89" s="4" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="O89" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2305.06090</t>
+          <t>https://arxiv.org/pdf/2607.25532</t>
         </is>
       </c>
     </row>
     <row r="90" ht="95" customHeight="1">
-      <c r="A90" s="12" t="inlineStr">
-        <is>
-          <t>BAPS</t>
+      <c r="A90" s="11" t="inlineStr">
+        <is>
+          <t>TabPFN-3</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Balanced Adaptive Prototype Selection for Scalable TabPFN Inference on Large-Scale Tabular Data</t>
+          <t>TabPFN-3: Technical Report</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr"/>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>사전학습된 표 형식 파운데이션 모델은 강력하지만 제한된 추론 문맥 길이 때문에 대규모 데이터셋 적용이 어렵다.</t>
+          <t>TabPFN이 표 형식 데이터의 파운데이션 모델 혁명을 이끌었지만, 기존 버전은 대규모 데이터셋 확장성과 학습·추론 속도에서 한계가 있었다.</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>모델 수정·재학습 없이 정보 보존형 압축 문맥을 구성하여 TabPFN을 백만 행 규모 데이터로 확장한다.</t>
+          <t>100만 학습 행까지 SOTA 성능을 확장하면서 학습·추론 시간을 대폭 줄인 차세대 표 형식 파운데이션 모델을 제시한다.</t>
         </is>
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>Balanced Adaptive Prototype Selection(BAPS)은 대표 구조, 결정 경계 정보, 국소 밀도, 클래스 균형, 특징 공간 다양성을 동시에 보존하는 프로토타입 선택으로 압축 문맥을 만든다. 사전학습 모델을 전혀 수정하지 않는 순수 문맥 구성 접근이다.</t>
+          <t>순수 합성 데이터만으로 사전학습된 차세대 PFN으로, 시계열·관계형·표-텍스트 데이터로 능력을 확장했다. 테스트타임 컴퓨트 스케일링을 도입하여 API 버전 TabPFN-3-Plus(Thinking)를 제공하고, SHAP 값 계산을 120배 가속하는 통합 기능을 갖췄다.</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr">
         <is>
-          <t>백만 행 규모의 HIGGS, SUSY 데이터셋</t>
+          <t>TabArena 벤치마크(최대 100만 행 데이터셋 포함), RelBench v1, TabSTAR, 시계열·표-텍스트 데이터</t>
         </is>
       </c>
       <c r="H90" s="4" t="inlineStr">
         <is>
-          <t>전체 데이터 문맥 및 기존 문맥 선택 방식 대비 예측 성능·캘리브레이션</t>
+          <t>기존 표 형식 모델 전체(GBDT 계열 포함), AutoGluon 1.5, TabPFN-2.5</t>
         </is>
       </c>
       <c r="I90" s="4" t="inlineStr">
         <is>
-          <t>512 프로토타입으로 압축한 문맥에서의 예측·캘리브레이션 평가, GPU 없이 Intel Core i7 CPU와 16GB RAM만으로 수행</t>
+          <t>TabArena Elo 비교, 대규모 서브셋 성능, 추론 속도 벤치마크, 관계형(RelBench)·표-텍스트 태스크 평가</t>
         </is>
       </c>
       <c r="J90" s="4" t="inlineStr">
         <is>
-          <t>predictive accuracy, calibration reliability, context compression ratio</t>
+          <t>Elo rating on TabArena, benchmark rank, training/inference time, SHAP computation speed</t>
         </is>
       </c>
       <c r="K90" s="4" t="inlineStr">
         <is>
-          <t>512개 프로토타입만으로 약 1,953배의 문맥 압축을 달성하면서 강한 예측 성능과 신뢰할 만한 캘리브레이션을 유지했고, GPU 없는 일반 CPU 환경에서 백만 행 데이터에 TabPFN을 적용할 수 있음을 보였다.</t>
+          <t>TabArena에서 단일 forward pass만으로 모든 타 모델을 큰 차이로 상회하고, TabPFN-3-Plus(Thinking)는 비-TabPFN 모델 대비 200 Elo 이상 우위이며 AutoGluon 1.5보다 10배 빠르다. TabPFN-2.5 대비 최대 20배 빠른 추론과 120배 빠른 SHAP 계산을 달성했다.</t>
         </is>
       </c>
       <c r="L90" s="4" t="inlineStr">
@@ -7115,7 +7096,7 @@
       </c>
       <c r="M90" s="4" t="inlineStr">
         <is>
-          <t>arXiv preprint</t>
+          <t>arXiv preprint (Prior Labs Technical Report)</t>
         </is>
       </c>
       <c r="N90" s="4" t="n">
@@ -7123,70 +7104,70 @@
       </c>
       <c r="O90" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2608.12989</t>
+          <t>https://arxiv.org/pdf/2605.13986</t>
         </is>
       </c>
     </row>
     <row r="91" ht="95" customHeight="1">
-      <c r="A91" s="12" t="inlineStr">
-        <is>
-          <t>ClusterAttn</t>
+      <c r="A91" s="11" t="inlineStr">
+        <is>
+          <t>TabPFN-Mech</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>ClusterAttention: A training-free speedup of bidirectional attention</t>
+          <t>Where Computation Lives Inside TabPFN: Causal Localisation of Attention Head Function</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr"/>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>TabPFN류 모델의 양방향 어텐션은 대규모 문맥에서 연산 병목이 되지만, 기존 희소 어텐션 가속 기법은 재학습이나 오프라인 캘리브레이션을 요구하거나 단일 패스 비정형 입력에 적용되지 못했다.</t>
+          <t>표 형식 파운데이션 모델의 내부 계산 메커니즘은 블랙박스로 남아 있으며, 어텐션 헤드들이 층별로 어떻게 계산을 분담하는지에 대한 인과적 분석이 전무했다.</t>
         </is>
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>재학습 없이 양방향 어텐션을 블록 희소화하여 TabPFN-3 추론을 가속한다.</t>
+          <t>TabPFN 2.5의 특징 단위 어텐션 헤드 기능을 인과적으로 국소화하는 최초의 기계론적(mechanistic) 분석을 수행한다.</t>
         </is>
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>각 어텐션 헤드의 key-query 기하에 적응하는 고속 재귀 클러스터링으로 블록 희소 어텐션을 구성하며, 클러스터 크기를 2의 거듭제곱으로 설정해 GPU에서 밀집 어텐션과 동일한 상호작용당 지연시간을 얻는다. 희소 어텐션 출력 오차의 해석적 표현을 유도해 조밀한 클러스터가 오히려 큰 오차를 낼 수 있음을 설명하고, 센트로이드 보상(centroid compensation)으로 이를 상쇄한다.</t>
+          <t>두 개의 합성 회귀 데이터셋에서 activation patching, ablation, 어텐션 엔트로피 분석을 결합해 헤드별 인과적 필요성을 측정한다. 추가로 contrastive activation steering을 통한 추론 시점 조종 가능성을 검증한다.</t>
         </is>
       </c>
       <c r="G91" s="4" t="inlineStr">
         <is>
-          <t>대규모 표 형식 데이터(TabPFN-3 추론), 비디오 생성(Wan 2.1-14B T2V)</t>
+          <t>통제된 합성 회귀 데이터셋 2종</t>
         </is>
       </c>
       <c r="H91" s="4" t="inlineStr">
         <is>
-          <t>밀집(dense) 어텐션, 선도적 어텐션 가속 기법들</t>
+          <t>헤드 간 인과 기여도 비교(patching vs ablation vs 엔트로피의 수렴 증거)</t>
         </is>
       </c>
       <c r="I91" s="4" t="inlineStr">
         <is>
-          <t>TabPFN-3 추론 가속 대 정확도 유지율 측정, 비디오 생성에서 기존 가속 기법과 출력 충실도-속도 비교</t>
+          <t>층별 activation patching·ablation으로 헤드 필요성 측정, 태스크 복잡도에 따른 지배 층 이동 분석, 샘플 간 steering 전이 실험</t>
         </is>
       </c>
       <c r="J91" s="4" t="inlineStr">
         <is>
-          <t>speedup factor, retained accuracy vs dense attention, output error</t>
+          <t>causal necessity (patching/ablation effect), attention entropy</t>
         </is>
       </c>
       <c r="K91" s="4" t="inlineStr">
         <is>
-          <t>TabPFN-3를 2~6배 가속하면서 밀집 어텐션 정확도의 99% 이상을 유지했으며, 단일 패스 비정형 입력에 성공적으로 적용된 최초의 training-free 어텐션 가속 기법이다. 비디오 생성에서도 기존 선도 기법보다 더 큰 가속으로 밀집 어텐션에 더 가까운 출력을 냈다.</t>
+          <t>한 헤드의 인과적 필요성이 피크 층에서 다른 헤드들의 2~5배로 지배적이고 그 지배 층이 태스크 복잡도에 따라 이동하는 시간적 특화를 발견했다. 반면 activation steering은 샘플 간 전이에 실패했는데, 이는 TabPFN이 LLM과 달리 안정적 파라미터 방향이 아닌 문맥 의존적 어텐션으로 태스크 구조를 인코딩하기 때문으로 해석된다.</t>
         </is>
       </c>
       <c r="L91" s="4" t="inlineStr">
         <is>
-          <t>명시 없음</t>
+          <t>합성 회귀 데이터셋 2종에 대한 분석으로 범위가 제한적이다.</t>
         </is>
       </c>
       <c r="M91" s="4" t="inlineStr">
         <is>
-          <t>arXiv preprint</t>
+          <t>FMSD Workshop @ ICML 2026</t>
         </is>
       </c>
       <c r="N91" s="4" t="n">
@@ -7194,65 +7175,65 @@
       </c>
       <c r="O91" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2608.26965</t>
+          <t>https://arxiv.org/pdf/2606.12917</t>
         </is>
       </c>
     </row>
     <row r="92" ht="95" customHeight="1">
-      <c r="A92" s="12" t="inlineStr">
-        <is>
-          <t>EnterpriseTab</t>
+      <c r="A92" s="11" t="inlineStr">
+        <is>
+          <t>TabPFN-MT</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Exploring Differences Between Tabular Enterprise Data and Public Benchmarks</t>
+          <t>TabPFN-MT: A Natively Multitask In-Context Learner for Tabular Data</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr"/>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>표 형식 모델과 벤치마크가 급증했지만 기업(enterprise) 데이터의 특성은 거의 연구되지 않았으며, 공개 벤치마크 성능이 실제 업무 데이터로 이어지는지 불분명하다.</t>
+          <t>PFN 계열은 표 형식 예측에서 성공했지만 단일 태스크 추론용으로 설계되어, 태스크 간 의존성을 활용하는 멀티태스크 학습에는 대응하지 못한다.</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>기업 표 형식 데이터의 통계적 특성을 분석하고 공개 벤치마크와의 성능 괴리를 실증한다.</t>
+          <t>다중 타깃 합성 prior로 학습하여 단일 forward pass로 멀티태스크 추론을 수행하는 표 형식 인컨텍스트 학습기를 만든다.</t>
         </is>
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>기업 데이터의 데이터 통계량을 공개 표 형식 벤치마크와 비교 분석하고, TabPFN·TabICL·ConTextTab 같은 표 형식 모델들의 성능을 양쪽에서 측정하여 일반화 여부를 검증한다.</t>
+          <t>다중 타깃으로 확장된 합성 prior에서 사전학습하여 문맥 내 태스크 간 의존성을 포착한다. 확장된 y-인코더와 공유 디코더 헤드를 사용해 그라디언트 학습 없이 멀티태스크 인컨텍스트 추론을 수행하며, 소규모-중규모 데이터셋에 특화되어 있다.</t>
         </is>
       </c>
       <c r="G92" s="4" t="inlineStr">
         <is>
-          <t>실제 기업(enterprise) 표 형식 데이터와 공개 표 형식 벤치마크</t>
+          <t>344개 데이터셋 (멀티태스크 표 형식 벤치마크)</t>
         </is>
       </c>
       <c r="H92" s="4" t="inlineStr">
         <is>
-          <t>TabPFN, TabICL, ConTextTab 등 표 형식 파운데이션 모델 간 및 데이터 소스 간 성능 비교</t>
+          <t>심층 표 형식 멀티태스크 학습 기법들, 최신 단일 태스크 앙상블</t>
         </is>
       </c>
       <c r="I92" s="4" t="inlineStr">
         <is>
-          <t>데이터 통계 특성 비교 분석, 동일 모델의 벤치마크 대 기업 데이터 성능 교차 측정</t>
+          <t>344개 데이터셋 대규모 평가, 단일 태스크 앙상블과의 컴퓨트 비대칭 비교, 추론 비용 분석</t>
         </is>
       </c>
       <c r="J92" s="4" t="inlineStr">
         <is>
-          <t>data statistics, model performance measurements across benchmark vs enterprise data</t>
+          <t>Accuracy rank, inference cost (forward passes)</t>
         </is>
       </c>
       <c r="K92" s="4" t="inlineStr">
         <is>
-          <t>기업 데이터는 공개 벤치마크와 뚜렷이 다르며, 전형적 벤치마크에서 잘하는 모델이 실제 기업 데이터에서 저조할 수 있고 그 역도 성립함을 보였다. 이는 기업급 특성을 가진 추가 벤치마크의 필요성을 시사한다.</t>
+          <t>멀티태스크 데이터셋에서 평균 Accuracy rank 4.89로 최고 순위를 기록하며 심층 표 형식 멀티태스크 학습의 새 SOTA를 세웠고, T개 태스크의 추론 비용을 O(T)에서 O(1) forward pass로 줄이면서 최신 단일 태스크 앙상블과도 대등했다.</t>
         </is>
       </c>
       <c r="L92" s="4" t="inlineStr">
         <is>
-          <t>기업 데이터의 비공개 특성상 재현 가능한 공개 벤치마크 제공에는 한계가 있다.</t>
+          <t>소규모-중규모 데이터셋에 특화되어 있다.</t>
         </is>
       </c>
       <c r="M92" s="4" t="inlineStr">
@@ -7265,74 +7246,70 @@
       </c>
       <c r="O92" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2606.30452</t>
+          <t>https://arxiv.org/pdf/2605.20234</t>
         </is>
       </c>
     </row>
     <row r="93" ht="95" customHeight="1">
-      <c r="A93" s="12" t="inlineStr">
-        <is>
-          <t>GOTabPFN</t>
+      <c r="A93" s="11" t="inlineStr">
+        <is>
+          <t>TabPFN-Rel</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>GOTabPFN: From Feature Ordering to Compact Tokenization for Tabular Foundation Models on High-Dimensional Data</t>
-        </is>
-      </c>
-      <c r="C93" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/zadid6pretam/GOTabPFN</t>
-        </is>
-      </c>
+          <t>Advancing Open and Reproducible Relational Learning: RelArena-α, TabPFN-Rel and RPI</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr"/>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>소형 표 형식 파운데이션 모델은 토큰 예산 제약 때문에 고차원-저표본(HDLSS) 데이터에서 성능이 불안정하며, 대형 백본 재학습 없이 이를 해결할 방법이 필요하다.</t>
+          <t>관계형 데이터베이스 학습(RelBench 등) 분야는 데이터 로딩·평가 프로토콜·튜닝 방식이 표준화되어 있지 않아 방법 간 공정 비교와 재현이 어렵다.</t>
         </is>
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
-          <t>특징 순서 최적화와 압축 토크나이제이션으로 재학습 없이 TabPFN류 모델을 고차원 데이터에 적용 가능하게 만든다.</t>
+          <t>관계형 학습을 위한 표준화 프레임워크, TabPFN-3 기반 관계형 하네스, 모델 불가지론적 인터페이스 3종을 오픈소스로 공개한다.</t>
         </is>
       </c>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>Graph-guided Ordering with Local Refinement(GO-LR)로 특징 순서를 최적화하며 이것이 가중 Minimum Linear Arrangement 문제와 동치임을 보인다. 이어 Neuro-Inspired Subunit Compression(NSC) 유닛이 국소적으로 인접한 정렬 특징들을 메타 특징으로 풀링하여 HDLSS 체제에 맞는 압축 표현을 만든다.</t>
+          <t>RelArena-α는 RelBench v1 베이스라인들의 데이터 로딩·평가·튜닝을 표준화한 통합 비교 프레임워크다. TabPFN-Rel은 TabPFN-3용 관계형 하네스로 RDBLearn을 개선한 것이며, RPI(Relational Predictive Interface)는 새 데이터베이스에 문제를 정의하고 임의 모델을 적용할 수 있는 모델 불가지론적 인터페이스다.</t>
         </is>
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>고차원-저표본(HDLSS) 특성의 표 형식 벤치마크들</t>
+          <t>RelBench v1 관계형 데이터베이스 벤치마크</t>
         </is>
       </c>
       <c r="H93" s="4" t="inlineStr">
         <is>
-          <t>특징 순서/압축을 적용하지 않은 TabPFN류 기본 모델 및 표 형식 베이스라인</t>
+          <t>RelBench v1의 그래프 신경망 등 특화 관계형 학습 방법들</t>
         </is>
       </c>
       <c r="I93" s="4" t="inlineStr">
         <is>
-          <t>타이트한 토큰 예산 하에서의 안정성·정확도 평가, 순서화-압축 구성요소 검증</t>
+          <t>RelArena-α 표준 프로토콜 하에서 RelBench v1 방법들과 TabPFN-Rel의 리더보드 비교</t>
         </is>
       </c>
       <c r="J93" s="4" t="inlineStr">
         <is>
-          <t>accuracy, stability under tight token budgets</t>
+          <t>RelArena-α leaderboard rank, RelBench task metrics</t>
         </is>
       </c>
       <c r="K93" s="4" t="inlineStr">
         <is>
-          <t>GOTabPFN이 타이트한 토큰 예산 조건에서 안정성과 정확도를 모두 개선하여, 백본 재학습 없이 소형 표 형식 파운데이션 모델을 고차원 데이터에 효과적으로 확장할 수 있음을 보였다.</t>
+          <t>TabPFN-Rel이 RelArena-α에서 1위를 기록하여, 관계형 데이터베이스를 평탄화(flattening)해 표 형식 파운데이션 모델에 넣는 접근이 특화 아키텍처와 여전히 경쟁력이 있음을 보였다.</t>
         </is>
       </c>
       <c r="L93" s="4" t="inlineStr">
         <is>
-          <t>명시 없음</t>
+          <t>α(초기) 버전 릴리스로 프레임워크와 인터페이스가 아직 초기 단계이다.</t>
         </is>
       </c>
       <c r="M93" s="4" t="inlineStr">
         <is>
-          <t>ICML 2026</t>
+          <t>arXiv preprint (Prior Labs)</t>
         </is>
       </c>
       <c r="N93" s="4" t="n">
@@ -7340,64 +7317,60 @@
       </c>
       <c r="O93" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2606.05441</t>
+          <t>https://arxiv.org/pdf/2608.16319</t>
         </is>
       </c>
     </row>
     <row r="94" ht="95" customHeight="1">
-      <c r="A94" s="12" t="inlineStr">
-        <is>
-          <t>LimiX-2M</t>
+      <c r="A94" s="11" t="inlineStr">
+        <is>
+          <t>TabSwift</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>LimiX-2M: Mitigating Low-Rank Collapse and Attention Bottlenecks in Tabular Foundation Models</t>
-        </is>
-      </c>
-      <c r="C94" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/limix-ldm-ai/LimiX</t>
-        </is>
-      </c>
+          <t>TabSwift: An Efficient Tabular Foundation Model with Row-Wise Attention</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr"/>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>표 형식 파운데이션 모델이 트리 앙상블에 필적하지만, 표준적인 affine 스칼라 토크나이제이션은 저층 표현의 저랭크 붕괴(low-rank collapse)와 어텐션 병목을 일으켜 연산 효율이 낮다.</t>
+          <t>최신 표 형식 파운데이션 모델들은 2차원(행+열) 어텐션으로 무거워졌는데, 원조 TabPFN식 경량 행 단위(row-wise) 어텐션 설계가 실제로 얼마나 경쟁력이 있는지 재검토가 필요하다.</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>값 인지 토크나이제이션과 계산 재배열로 소형 모델의 정확도-효율 트레이드오프를 개선한다.</t>
+          <t>행 단위 어텐션만으로 강력한 표 형식 파운데이션 모델과 대등하면서 추론이 훨씬 효율적인 모델을 설계한다.</t>
         </is>
       </c>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>통합 tokenize-and-route 프레임워크를 제안한다. RaBEL이 각 스칼라 값을 국소화된 RBF 특징으로 확장해 조건화와 얕은 층의 유효 랭크를 개선하고, 양방향 블록을 S→N→F 순서로 재배열해 계산을 readout에 정렬시킨다.</t>
+          <t>행 단위 어텐션 전용 백본에 게이트 어텐션 안정화 메커니즘과 소수의 학습 가능한 레지스터 토큰(전역 문맥 제공)을 결합한다. 분류·회귀를 모두 지원하며, 샘플별로 추론 깊이를 동적으로 조절하는 적응적 층별 조기 종료(early-exit) 메커니즘으로 anytime 추론을 가능케 한다.</t>
         </is>
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
-          <t>널리 쓰이는 표 형식 벤치마크들</t>
+          <t>표 형식 분류·회귀 벤치마크 (초록에 세부 명시 없음)</t>
         </is>
       </c>
       <c r="H94" s="4" t="inlineStr">
         <is>
-          <t>더 큰 규모의 TabPFN-v2, TabICL</t>
+          <t>TabPFN v2, TabICL 등 더 강력한 표 형식 파운데이션 모델</t>
         </is>
       </c>
       <c r="I94" s="4" t="inlineStr">
         <is>
-          <t>벤치마크 정확도 비교와 학습·추론 비용 분석, 토크나이제이션·블록 순서 설계 검증</t>
+          <t>파운데이션 모델 대비 성능·추론 효율 비교, 조기 종료 메커니즘 검증</t>
         </is>
       </c>
       <c r="J94" s="4" t="inlineStr">
         <is>
-          <t>benchmark accuracy/rank, training and inference cost, effective rank</t>
+          <t>classification/regression accuracy, inference efficiency (latency/depth)</t>
         </is>
       </c>
       <c r="K94" s="4" t="inlineStr">
         <is>
-          <t>단 2M 파라미터의 LimiX-2M이 자신보다 큰 TabPFN-v2와 TabICL을 표 형식 벤치마크에서 상회하면서 학습·추론 비용을 동시에 절감했다.</t>
+          <t>경량 행 단위 어텐션 백본이 더 강한 표 형식 파운데이션 모델들과 경쟁력을 유지하면서 추론 효율이 훨씬 높고, 적응적 조기 종료로 실용 배포에 적합한 anytime 인컨텍스트 학습을 달성했다 (ICML 2026 spotlight).</t>
         </is>
       </c>
       <c r="L94" s="4" t="inlineStr">
@@ -7407,7 +7380,7 @@
       </c>
       <c r="M94" s="4" t="inlineStr">
         <is>
-          <t>ICML 2026</t>
+          <t>ICML 2026 (spotlight)</t>
         </is>
       </c>
       <c r="N94" s="4" t="n">
@@ -7415,597 +7388,12 @@
       </c>
       <c r="O94" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/pdf/2606.04485</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="95" customHeight="1">
-      <c r="A95" s="12" t="inlineStr">
-        <is>
-          <t>SpurRoute</t>
-        </is>
-      </c>
-      <c r="B95" s="4" t="inlineStr">
-        <is>
-          <t>Entangled by Design: Spurious Intra-Variable Signal Routing in Tabular In-Context Learners</t>
-        </is>
-      </c>
-      <c r="C95" s="4" t="inlineStr"/>
-      <c r="D95" s="4" t="inlineStr">
-        <is>
-          <t>하나의 특징이 진짜 인과 신호와 장비 아티팩트 같은 허위 신호를 함께 담고 있을 때(예: 병원별 측정 장비 편향), 인컨텍스트 학습기는 허위 신호를 통해 예측을 라우팅하여 새 환경에서 조용히 실패할 수 있다.</t>
-        </is>
-      </c>
-      <c r="E95" s="4" t="inlineStr">
-        <is>
-          <t>표 형식 인컨텍스트 학습기의 변수 내 허위 신호 라우팅을 이론적으로 정식화하고 경량 완화책을 제시한다.</t>
-        </is>
-      </c>
-      <c r="F95" s="4" t="inlineStr">
-        <is>
-          <t>X=[C; αS; η] 형태의 복합 표현에서 ridge ICL이 문맥 크기와 무관하게 허위 라우팅을 피할 수 없음을 증명하고, CSR ∝ ρ_S/ρ_C의 닫힌 형식 특성화를 유도한다. 약한 환경 라벨만 요구하는 두 가지 완화책(환경 층화 문맥 구성, S-swap 증강)을 제안한다.</t>
-        </is>
-      </c>
-      <c r="G95" s="4" t="inlineStr">
-        <is>
-          <t>인과/허위 신호 부분공간을 통제한 합성 복합 표현 데이터</t>
-        </is>
-      </c>
-      <c r="H95" s="4" t="inlineStr">
-        <is>
-          <t>선형(ridge) ICL 이론 예측 vs TabPFN의 실증 거동</t>
-        </is>
-      </c>
-      <c r="I95" s="4" t="inlineStr">
-        <is>
-          <t>닫힌 형식 예측의 실증 검증, 문맥 크기에 따른 허위 라우팅 증폭 측정, 완화책 적용 전후 CSR 비교</t>
-        </is>
-      </c>
-      <c r="J95" s="4" t="inlineStr">
-        <is>
-          <t>Causal-Spurious Routing ratio (CSR), correlation with closed-form prediction, causal sensitivity</t>
-        </is>
-      </c>
-      <c r="K95" s="4" t="inlineStr">
-        <is>
-          <t>닫힌 형식 특성화가 선형 ICL에서 r=0.997, TabPFN에서 r=0.979로 확인되었고, 직관과 달리 문맥이 클수록 허위 라우팅이 최대 1.74배 증폭되었다. S-swap 증강은 허위 라우팅을 선형 ICL에서 74%, TabPFN에서 98.8% 줄이면서 TabPFN의 인과 민감도를 8.4배 높였다.</t>
-        </is>
-      </c>
-      <c r="L95" s="4" t="inlineStr">
-        <is>
-          <t>명시 없음</t>
-        </is>
-      </c>
-      <c r="M95" s="4" t="inlineStr">
-        <is>
-          <t>arXiv preprint</t>
-        </is>
-      </c>
-      <c r="N95" s="4" t="n">
-        <v>2026</v>
-      </c>
-      <c r="O95" s="4" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/pdf/2607.25532</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="95" customHeight="1">
-      <c r="A96" s="12" t="inlineStr">
-        <is>
-          <t>TabPFN-3</t>
-        </is>
-      </c>
-      <c r="B96" s="4" t="inlineStr">
-        <is>
-          <t>TabPFN-3: Technical Report</t>
-        </is>
-      </c>
-      <c r="C96" s="4" t="inlineStr"/>
-      <c r="D96" s="4" t="inlineStr">
-        <is>
-          <t>TabPFN이 표 형식 데이터의 파운데이션 모델 혁명을 이끌었지만, 기존 버전은 대규모 데이터셋 확장성과 학습·추론 속도에서 한계가 있었다.</t>
-        </is>
-      </c>
-      <c r="E96" s="4" t="inlineStr">
-        <is>
-          <t>100만 학습 행까지 SOTA 성능을 확장하면서 학습·추론 시간을 대폭 줄인 차세대 표 형식 파운데이션 모델을 제시한다.</t>
-        </is>
-      </c>
-      <c r="F96" s="4" t="inlineStr">
-        <is>
-          <t>순수 합성 데이터만으로 사전학습된 차세대 PFN으로, 시계열·관계형·표-텍스트 데이터로 능력을 확장했다. 테스트타임 컴퓨트 스케일링을 도입하여 API 버전 TabPFN-3-Plus(Thinking)를 제공하고, SHAP 값 계산을 120배 가속하는 통합 기능을 갖췄다.</t>
-        </is>
-      </c>
-      <c r="G96" s="4" t="inlineStr">
-        <is>
-          <t>TabArena 벤치마크(최대 100만 행 데이터셋 포함), RelBench v1, TabSTAR, 시계열·표-텍스트 데이터</t>
-        </is>
-      </c>
-      <c r="H96" s="4" t="inlineStr">
-        <is>
-          <t>기존 표 형식 모델 전체(GBDT 계열 포함), AutoGluon 1.5, TabPFN-2.5</t>
-        </is>
-      </c>
-      <c r="I96" s="4" t="inlineStr">
-        <is>
-          <t>TabArena Elo 비교, 대규모 서브셋 성능, 추론 속도 벤치마크, 관계형(RelBench)·표-텍스트 태스크 평가</t>
-        </is>
-      </c>
-      <c r="J96" s="4" t="inlineStr">
-        <is>
-          <t>Elo rating on TabArena, benchmark rank, training/inference time, SHAP computation speed</t>
-        </is>
-      </c>
-      <c r="K96" s="4" t="inlineStr">
-        <is>
-          <t>TabArena에서 단일 forward pass만으로 모든 타 모델을 큰 차이로 상회하고, TabPFN-3-Plus(Thinking)는 비-TabPFN 모델 대비 200 Elo 이상 우위이며 AutoGluon 1.5보다 10배 빠르다. TabPFN-2.5 대비 최대 20배 빠른 추론과 120배 빠른 SHAP 계산을 달성했다.</t>
-        </is>
-      </c>
-      <c r="L96" s="4" t="inlineStr">
-        <is>
-          <t>명시 없음</t>
-        </is>
-      </c>
-      <c r="M96" s="4" t="inlineStr">
-        <is>
-          <t>arXiv preprint (Prior Labs Technical Report)</t>
-        </is>
-      </c>
-      <c r="N96" s="4" t="n">
-        <v>2026</v>
-      </c>
-      <c r="O96" s="4" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/pdf/2605.13986</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="95" customHeight="1">
-      <c r="A97" s="12" t="inlineStr">
-        <is>
-          <t>TabPFN-Mech</t>
-        </is>
-      </c>
-      <c r="B97" s="4" t="inlineStr">
-        <is>
-          <t>Where Computation Lives Inside TabPFN: Causal Localisation of Attention Head Function</t>
-        </is>
-      </c>
-      <c r="C97" s="4" t="inlineStr"/>
-      <c r="D97" s="4" t="inlineStr">
-        <is>
-          <t>표 형식 파운데이션 모델의 내부 계산 메커니즘은 블랙박스로 남아 있으며, 어텐션 헤드들이 층별로 어떻게 계산을 분담하는지에 대한 인과적 분석이 전무했다.</t>
-        </is>
-      </c>
-      <c r="E97" s="4" t="inlineStr">
-        <is>
-          <t>TabPFN 2.5의 특징 단위 어텐션 헤드 기능을 인과적으로 국소화하는 최초의 기계론적(mechanistic) 분석을 수행한다.</t>
-        </is>
-      </c>
-      <c r="F97" s="4" t="inlineStr">
-        <is>
-          <t>두 개의 합성 회귀 데이터셋에서 activation patching, ablation, 어텐션 엔트로피 분석을 결합해 헤드별 인과적 필요성을 측정한다. 추가로 contrastive activation steering을 통한 추론 시점 조종 가능성을 검증한다.</t>
-        </is>
-      </c>
-      <c r="G97" s="4" t="inlineStr">
-        <is>
-          <t>통제된 합성 회귀 데이터셋 2종</t>
-        </is>
-      </c>
-      <c r="H97" s="4" t="inlineStr">
-        <is>
-          <t>헤드 간 인과 기여도 비교(patching vs ablation vs 엔트로피의 수렴 증거)</t>
-        </is>
-      </c>
-      <c r="I97" s="4" t="inlineStr">
-        <is>
-          <t>층별 activation patching·ablation으로 헤드 필요성 측정, 태스크 복잡도에 따른 지배 층 이동 분석, 샘플 간 steering 전이 실험</t>
-        </is>
-      </c>
-      <c r="J97" s="4" t="inlineStr">
-        <is>
-          <t>causal necessity (patching/ablation effect), attention entropy</t>
-        </is>
-      </c>
-      <c r="K97" s="4" t="inlineStr">
-        <is>
-          <t>한 헤드의 인과적 필요성이 피크 층에서 다른 헤드들의 2~5배로 지배적이고 그 지배 층이 태스크 복잡도에 따라 이동하는 시간적 특화를 발견했다. 반면 activation steering은 샘플 간 전이에 실패했는데, 이는 TabPFN이 LLM과 달리 안정적 파라미터 방향이 아닌 문맥 의존적 어텐션으로 태스크 구조를 인코딩하기 때문으로 해석된다.</t>
-        </is>
-      </c>
-      <c r="L97" s="4" t="inlineStr">
-        <is>
-          <t>합성 회귀 데이터셋 2종에 대한 분석으로 범위가 제한적이다.</t>
-        </is>
-      </c>
-      <c r="M97" s="4" t="inlineStr">
-        <is>
-          <t>FMSD Workshop @ ICML 2026</t>
-        </is>
-      </c>
-      <c r="N97" s="4" t="n">
-        <v>2026</v>
-      </c>
-      <c r="O97" s="4" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/pdf/2606.12917</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="95" customHeight="1">
-      <c r="A98" s="12" t="inlineStr">
-        <is>
-          <t>TabPFN-MT</t>
-        </is>
-      </c>
-      <c r="B98" s="4" t="inlineStr">
-        <is>
-          <t>TabPFN-MT: A Natively Multitask In-Context Learner for Tabular Data</t>
-        </is>
-      </c>
-      <c r="C98" s="4" t="inlineStr"/>
-      <c r="D98" s="4" t="inlineStr">
-        <is>
-          <t>PFN 계열은 표 형식 예측에서 성공했지만 단일 태스크 추론용으로 설계되어, 태스크 간 의존성을 활용하는 멀티태스크 학습에는 대응하지 못한다.</t>
-        </is>
-      </c>
-      <c r="E98" s="4" t="inlineStr">
-        <is>
-          <t>다중 타깃 합성 prior로 학습하여 단일 forward pass로 멀티태스크 추론을 수행하는 표 형식 인컨텍스트 학습기를 만든다.</t>
-        </is>
-      </c>
-      <c r="F98" s="4" t="inlineStr">
-        <is>
-          <t>다중 타깃으로 확장된 합성 prior에서 사전학습하여 문맥 내 태스크 간 의존성을 포착한다. 확장된 y-인코더와 공유 디코더 헤드를 사용해 그라디언트 학습 없이 멀티태스크 인컨텍스트 추론을 수행하며, 소규모-중규모 데이터셋에 특화되어 있다.</t>
-        </is>
-      </c>
-      <c r="G98" s="4" t="inlineStr">
-        <is>
-          <t>344개 데이터셋 (멀티태스크 표 형식 벤치마크)</t>
-        </is>
-      </c>
-      <c r="H98" s="4" t="inlineStr">
-        <is>
-          <t>심층 표 형식 멀티태스크 학습 기법들, 최신 단일 태스크 앙상블</t>
-        </is>
-      </c>
-      <c r="I98" s="4" t="inlineStr">
-        <is>
-          <t>344개 데이터셋 대규모 평가, 단일 태스크 앙상블과의 컴퓨트 비대칭 비교, 추론 비용 분석</t>
-        </is>
-      </c>
-      <c r="J98" s="4" t="inlineStr">
-        <is>
-          <t>Accuracy rank, inference cost (forward passes)</t>
-        </is>
-      </c>
-      <c r="K98" s="4" t="inlineStr">
-        <is>
-          <t>멀티태스크 데이터셋에서 평균 Accuracy rank 4.89로 최고 순위를 기록하며 심층 표 형식 멀티태스크 학습의 새 SOTA를 세웠고, T개 태스크의 추론 비용을 O(T)에서 O(1) forward pass로 줄이면서 최신 단일 태스크 앙상블과도 대등했다.</t>
-        </is>
-      </c>
-      <c r="L98" s="4" t="inlineStr">
-        <is>
-          <t>소규모-중규모 데이터셋에 특화되어 있다.</t>
-        </is>
-      </c>
-      <c r="M98" s="4" t="inlineStr">
-        <is>
-          <t>arXiv preprint</t>
-        </is>
-      </c>
-      <c r="N98" s="4" t="n">
-        <v>2026</v>
-      </c>
-      <c r="O98" s="4" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/pdf/2605.20234</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="95" customHeight="1">
-      <c r="A99" s="12" t="inlineStr">
-        <is>
-          <t>TabPFN-Rel</t>
-        </is>
-      </c>
-      <c r="B99" s="4" t="inlineStr">
-        <is>
-          <t>Advancing Open and Reproducible Relational Learning: RelArena-α, TabPFN-Rel and RPI</t>
-        </is>
-      </c>
-      <c r="C99" s="4" t="inlineStr"/>
-      <c r="D99" s="4" t="inlineStr">
-        <is>
-          <t>관계형 데이터베이스 학습(RelBench 등) 분야는 데이터 로딩·평가 프로토콜·튜닝 방식이 표준화되어 있지 않아 방법 간 공정 비교와 재현이 어렵다.</t>
-        </is>
-      </c>
-      <c r="E99" s="4" t="inlineStr">
-        <is>
-          <t>관계형 학습을 위한 표준화 프레임워크, TabPFN-3 기반 관계형 하네스, 모델 불가지론적 인터페이스 3종을 오픈소스로 공개한다.</t>
-        </is>
-      </c>
-      <c r="F99" s="4" t="inlineStr">
-        <is>
-          <t>RelArena-α는 RelBench v1 베이스라인들의 데이터 로딩·평가·튜닝을 표준화한 통합 비교 프레임워크다. TabPFN-Rel은 TabPFN-3용 관계형 하네스로 RDBLearn을 개선한 것이며, RPI(Relational Predictive Interface)는 새 데이터베이스에 문제를 정의하고 임의 모델을 적용할 수 있는 모델 불가지론적 인터페이스다.</t>
-        </is>
-      </c>
-      <c r="G99" s="4" t="inlineStr">
-        <is>
-          <t>RelBench v1 관계형 데이터베이스 벤치마크</t>
-        </is>
-      </c>
-      <c r="H99" s="4" t="inlineStr">
-        <is>
-          <t>RelBench v1의 그래프 신경망 등 특화 관계형 학습 방법들</t>
-        </is>
-      </c>
-      <c r="I99" s="4" t="inlineStr">
-        <is>
-          <t>RelArena-α 표준 프로토콜 하에서 RelBench v1 방법들과 TabPFN-Rel의 리더보드 비교</t>
-        </is>
-      </c>
-      <c r="J99" s="4" t="inlineStr">
-        <is>
-          <t>RelArena-α leaderboard rank, RelBench task metrics</t>
-        </is>
-      </c>
-      <c r="K99" s="4" t="inlineStr">
-        <is>
-          <t>TabPFN-Rel이 RelArena-α에서 1위를 기록하여, 관계형 데이터베이스를 평탄화(flattening)해 표 형식 파운데이션 모델에 넣는 접근이 특화 아키텍처와 여전히 경쟁력이 있음을 보였다.</t>
-        </is>
-      </c>
-      <c r="L99" s="4" t="inlineStr">
-        <is>
-          <t>α(초기) 버전 릴리스로 프레임워크와 인터페이스가 아직 초기 단계이다.</t>
-        </is>
-      </c>
-      <c r="M99" s="4" t="inlineStr">
-        <is>
-          <t>arXiv preprint (Prior Labs)</t>
-        </is>
-      </c>
-      <c r="N99" s="4" t="n">
-        <v>2026</v>
-      </c>
-      <c r="O99" s="4" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/pdf/2608.16319</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="95" customHeight="1">
-      <c r="A100" s="12" t="inlineStr">
-        <is>
-          <t>TabSwift</t>
-        </is>
-      </c>
-      <c r="B100" s="4" t="inlineStr">
-        <is>
-          <t>TabSwift: An Efficient Tabular Foundation Model with Row-Wise Attention</t>
-        </is>
-      </c>
-      <c r="C100" s="4" t="inlineStr"/>
-      <c r="D100" s="4" t="inlineStr">
-        <is>
-          <t>최신 표 형식 파운데이션 모델들은 2차원(행+열) 어텐션으로 무거워졌는데, 원조 TabPFN식 경량 행 단위(row-wise) 어텐션 설계가 실제로 얼마나 경쟁력이 있는지 재검토가 필요하다.</t>
-        </is>
-      </c>
-      <c r="E100" s="4" t="inlineStr">
-        <is>
-          <t>행 단위 어텐션만으로 강력한 표 형식 파운데이션 모델과 대등하면서 추론이 훨씬 효율적인 모델을 설계한다.</t>
-        </is>
-      </c>
-      <c r="F100" s="4" t="inlineStr">
-        <is>
-          <t>행 단위 어텐션 전용 백본에 게이트 어텐션 안정화 메커니즘과 소수의 학습 가능한 레지스터 토큰(전역 문맥 제공)을 결합한다. 분류·회귀를 모두 지원하며, 샘플별로 추론 깊이를 동적으로 조절하는 적응적 층별 조기 종료(early-exit) 메커니즘으로 anytime 추론을 가능케 한다.</t>
-        </is>
-      </c>
-      <c r="G100" s="4" t="inlineStr">
-        <is>
-          <t>표 형식 분류·회귀 벤치마크 (초록에 세부 명시 없음)</t>
-        </is>
-      </c>
-      <c r="H100" s="4" t="inlineStr">
-        <is>
-          <t>TabPFN v2, TabICL 등 더 강력한 표 형식 파운데이션 모델</t>
-        </is>
-      </c>
-      <c r="I100" s="4" t="inlineStr">
-        <is>
-          <t>파운데이션 모델 대비 성능·추론 효율 비교, 조기 종료 메커니즘 검증</t>
-        </is>
-      </c>
-      <c r="J100" s="4" t="inlineStr">
-        <is>
-          <t>classification/regression accuracy, inference efficiency (latency/depth)</t>
-        </is>
-      </c>
-      <c r="K100" s="4" t="inlineStr">
-        <is>
-          <t>경량 행 단위 어텐션 백본이 더 강한 표 형식 파운데이션 모델들과 경쟁력을 유지하면서 추론 효율이 훨씬 높고, 적응적 조기 종료로 실용 배포에 적합한 anytime 인컨텍스트 학습을 달성했다 (ICML 2026 spotlight).</t>
-        </is>
-      </c>
-      <c r="L100" s="4" t="inlineStr">
-        <is>
-          <t>명시 없음</t>
-        </is>
-      </c>
-      <c r="M100" s="4" t="inlineStr">
-        <is>
-          <t>ICML 2026 (spotlight)</t>
-        </is>
-      </c>
-      <c r="N100" s="4" t="n">
-        <v>2026</v>
-      </c>
-      <c r="O100" s="4" t="inlineStr">
-        <is>
           <t>https://arxiv.org/pdf/2606.07345</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O100"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="13" t="inlineStr">
-        <is>
-          <t>행 순서(그룹)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="14" t="inlineStr">
-        <is>
-          <t>교수님 추가</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>3편</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>imbalance(기존 22편 재정리)</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>21편</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="16" t="inlineStr">
-        <is>
-          <t>TabPFN core/버전</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>12편</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="17" t="inlineStr">
-        <is>
-          <t>context/retrieval/scaling</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>8편</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>finetuning/적응</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>8편</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>생성/증강/결측</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>8편</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="20" t="inlineStr">
-        <is>
-          <t>이론/분석/벤치마크</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>10편</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="21" t="inlineStr">
-        <is>
-          <t>도메인 응용</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>6편</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="22" t="inlineStr">
-        <is>
-          <t>인접 tabular FM</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>12편</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="23" t="inlineStr">
-        <is>
-          <t>2026 최신</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>11편</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>주의</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>노란 행 = 교수님 추가 3편. Abb. 셀 색 = 그룹. "(스니펫 검증)" = 초록 원문 접근 차단으로 검색 스니펫 기반. 모든 항목은 초록 페이지 실확인 후 수록.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <autoFilter ref="A1:O94"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>